<commit_message>
Reconcile 97 policy records with primary sources and synced exports
</commit_message>
<xml_diff>
--- a/public/levantamentos/politicas-ia/base-politicas-ia-2026-10.xlsx
+++ b/public/levantamentos/politicas-ia/base-politicas-ia-2026-10.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="1" r:id="Rcf983fc792414fbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livro de códigos" sheetId="2" r:id="R3e0b62411b984c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="1" r:id="Re7101c99ab2c4398"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livro de códigos" sheetId="2" r:id="Ra2cef9c784da49b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,13 +55,16 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -568,9 +571,7 @@
       <x:c r="E3" t="str">
         <x:v>Internacional</x:v>
       </x:c>
-      <x:c r="F3" t="n">
-        <x:v>2023</x:v>
-      </x:c>
+      <x:c r="F3"/>
       <x:c r="G3" t="str">
         <x:v>Permitida</x:v>
       </x:c>
@@ -590,7 +591,7 @@
         <x:v>https://www.icmje.org/recommendations/browse/artificial-intelligence/ai-use-by-authors.html</x:v>
       </x:c>
       <x:c r="M3" t="str">
-        <x:v>Declarar na carta e no trabalho; IA não é fonte primária.</x:v>
+        <x:v>As recomendações distinguem autoria, parecer e edição. Autores devem declarar o uso na carta de apresentação e na seção pertinente do manuscrito, verificar exatidão, plágio e referências; IA não é autora nem fonte primária. Pareceristas seguem a política do periódico ou pedem autorização prévia e declaram o uso. Manuscritos não podem ser enviados a sistemas sem confidencialidade assegurada salvo a permissão expressa aplicável. O texto inclui imagens na responsabilidade autoral, mas não estabelece aqui uma política específica de permissão de imagens. Ano da versão consultada não explicitado.</x:v>
       </x:c>
       <x:c r="N3" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -665,7 +666,7 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H5" t="str">
-        <x:v>Submissão/carta</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I5" t="str">
         <x:v>Condicionado</x:v>
@@ -677,10 +678,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L5" t="str">
-        <x:v>https://www.cse-scienceeditor.org/article/cse-guidance-on-machine-learning-and-artificial-intelligence-tools/</x:v>
+        <x:v>https://www.councilscienceeditors.org/2-1-editor-roles-and-responsibilities</x:v>
       </x:c>
       <x:c r="M5" t="str">
-        <x:v>Guia 2023: declarar em pergunta da submissão ou na carta. Recomendações §2.1.15 (atualiz. 26/12/2025): declarar na submissão inicial; nenhuma parte de manuscrito ou parecer em chatbot público.</x:v>
+        <x:v>Seção 2.1.15 atualizada em 26 de dezembro de 2025. Recomenda políticas explícitas e revisão anual; autores, revisores e editores devem divulgar ferramenta e finalidade, exceto usos básicos de gramática/ortografia. Autores declaram na submissão ao periódico e aos leitores, com responsabilidade integral. Nenhuma parte do manuscrito ou parecer pode ser inserida em chatbot/LLM público; decisões editoriais não podem depender apenas de sínteses/recomendações geradas. Recomenda que cada periódico especifique regras para texto, imagens e demais usos; não estabelece permissão universal de imagens.</x:v>
       </x:c>
       <x:c r="N5" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -817,7 +818,7 @@
         <x:v>https://research-and-innovation.ec.europa.eu/document/download/2b6cf7e5-36ac-41cb-aab5-0d32050143dc_en?filename=ec_rtd_ai-guidelines.pdf</x:v>
       </x:c>
       <x:c r="M8" t="str">
-        <x:v>3ª versão (maio/2026); evitar uso substancial em revisão; alerta para prompts ocultos.</x:v>
+        <x:v>Quarta edição, outubro de 2026. Diretrizes de responsabilidade e transparência, sem criar novos requisitos legais. Pesquisadores permanecem responsáveis e devem declarar usos substanciais conforme as regras disciplinares, editoriais, institucionais e de fomento; correção técnica menor geralmente dispensa declaração. Na avaliação, apoio limitado somente quando autorizado: pode esclarecer conceitos ou linguagem, mas não redigir pareceres nem avaliar mérito científico. Não fixa seção universal de declaração nem regra específica de imagens.</x:v>
       </x:c>
       <x:c r="N8" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -859,10 +860,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L9" t="str">
-        <x:v>https://niso.org/niso-io/2025/09/stm-releases-recommendations-classification-ai-use-manuscript-preparation</x:v>
+        <x:v>https://s3.eu-west-2.amazonaws.com/stm.offloadmedia/wp-content/uploads/2025/04/23020709/STM_AI_Classification_Recs_19_Sept2025-1.pdf</x:v>
       </x:c>
       <x:c r="M9" t="str">
-        <x:v>9 categorias; não fixa regras.</x:v>
+        <x:v>Quadro final de setembro de 2025 com nove classes de uso na preparação de manuscritos. Distingue redação, tradução, formatação de dados/código, ilustração, visualização e referências. Não harmoniza nem determina permissões ou locais de declaração: essas decisões cabem às editoras e comunidades. Não regula uso de IA como método de pesquisa nem fornece norma própria de pareceristas. Identificar um uso na classificação não significa autorizá-lo.</x:v>
       </x:c>
       <x:c r="N9" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -905,7 +906,7 @@
         <x:v>https://www.lib.szu.edu.cn/sites/szulib/files/2025-06/%E5%AD%A6%E6%9C%AF%E5%87%BA%E7%89%88%E4%B8%ADAIGC%E4%BD%BF%E7%94%A8%E8%BE%B9%E7%95%8C%E6%8C%87%E5%8D%972.0.pdf</x:v>
       </x:c>
       <x:c r="M10" t="str">
-        <x:v>Veda gerar hipóteses, artigo inteiro e conclusões; exige prompts na declaração.</x:v>
+        <x:v>Guia AIGC 2.0 elaborado pelo ISTIC com editoras parceiras; não substitui a política individual de cada editora/periódico. Admite apoio à redação e apresentação de dados reais, sob responsabilidade humana, e pede descrição de ferramenta, versão, usos e partes afetadas em Métodos ou Agradecimentos. Pareceristas só podem usar apoio permitido pela revista, sem enviar manuscritos confidenciais à ferramenta. Proíbe fabricar imagens experimentais e usar IA em resumos gráficos; arte de capa exige autorização prévia e direitos. Ano normativo não explicitado no documento consultado.</x:v>
       </x:c>
       <x:c r="N10" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -1173,7 +1174,7 @@
         <x:v>https://www.amstat.org/docs/default-source/amstat-documents/asa-statement-on-ethical-ai-principles-for-statistical-practitioners.pdf</x:v>
       </x:c>
       <x:c r="M16" t="str">
-        <x:v>Princípios éticos; sem regra de autoria.</x:v>
+        <x:v>Declaração de 8 de outubro de 2024 sobre responsabilidade, transparência e equidade no desenvolvimento e uso de IA por profissionais de estatística. Não estabelece neste documento uma regra editorial de autoria, local de declaração, pareceres ou imagens; remete a orientações mais específicas para publicações. A codificação de ausência se limita à fonte examinada, não a todos os periódicos associados.</x:v>
       </x:c>
       <x:c r="N16" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -1286,14 +1287,12 @@
       <x:c r="E19" t="str">
         <x:v>Internacional</x:v>
       </x:c>
-      <x:c r="F19" t="n">
-        <x:v>2023</x:v>
-      </x:c>
+      <x:c r="F19"/>
       <x:c r="G19" t="str">
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H19" t="str">
-        <x:v>Não especifica</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I19" t="str">
         <x:v>Condicionado</x:v>
@@ -1305,10 +1304,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L19" t="str">
-        <x:v>https://2023.aclweb.org/blog/ACL-2023-policy/</x:v>
+        <x:v>https://www.aclweb.org/adminwiki/index.php/ACL_Policy_on_Publication_Ethics</x:v>
       </x:c>
       <x:c r="M19" t="str">
-        <x:v>Espectro de usos; revisores não geram 1º rascunho.</x:v>
+        <x:v>Política central vigente: IA não é autora; usos de geração de conteúdo, inclusive réplicas, devem ser apropriados e declarados em Agradecimentos, com verificação e atribuição. Correção simples de linguagem e sugestões curtas dispensam. No ARR, também informar no Responsible NLP Checklist; código pode ser documentado no README. Pareceristas leem integralmente e escrevem o próprio primeiro rascunho e argumentos; podem obter apoio responsável de linguagem ou provas, mas não enviar manuscritos ou pareceres a ferramentas sem privacidade. Sem norma específica de imagens nesta seção; consultar exigências da trilha.</x:v>
       </x:c>
       <x:c r="N19" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -1332,7 +1331,7 @@
         <x:v>Internacional</x:v>
       </x:c>
       <x:c r="F20" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="G20" t="str">
         <x:v>Permitida</x:v>
@@ -1350,10 +1349,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L20" t="str">
-        <x:v>https://neurips.cc/Conferences/2025/LLM</x:v>
+        <x:v>https://neurips.cc/Conferences/2026/MainTrackHandbook</x:v>
       </x:c>
       <x:c r="M20" t="str">
-        <x:v>LLM como método no setup experimental.</x:v>
+        <x:v>Main Track 2026: autores podem usar ferramentas sob responsabilidade integral; agentes/LLMs como componente metodológico importante, original ou não padrão devem ser descritos no desenho experimental/equivalente. Correções linguísticas e apoio básico de código dispensam relato. Pareceristas só podem usar o LLM autorizado via OpenReview nos artigos especificamente elegíveis ao experimento; nos demais, não. A confidencialidade permanece obrigatória. Outras trilhas e workshops têm regras distintas, inclusive restrições de redação; a regra não é universal para todo o evento.</x:v>
       </x:c>
       <x:c r="N20" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -1395,10 +1394,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L21" t="str">
-        <x:v>https://blog.icml.cc/?p=1167</x:v>
+        <x:v>https://icml.cc/Conferences/2026/LLM-Policy</x:v>
       </x:c>
       <x:c r="M21" t="str">
-        <x:v>Políticas A/B; 497 artigos rejeitados por revisores infratores.</x:v>
+        <x:v>ICML 2026 admite IA na escrita/pesquisa sob responsabilidade dos autores e incentiva explicar usos metodológicos relevantes; não fixa declaração universal para redação. Não admite IA como autora e proíbe prompt injection. Revisão: A proíbe LLMs, com exceção de uso inadvertido em ferramentas tradicionais; B permite compreensão, busca de trabalhos e polimento em sistemas com privacidade, mas não delegar crítica, resumir o artigo ou redigir o parecer. Autor e revisor são vinculados ao regime atribuído. Não há nesta norma regra específica de imagens.</x:v>
       </x:c>
       <x:c r="N21" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -2083,7 +2082,7 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H37" t="str">
-        <x:v>Seção própria</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I37" t="str">
         <x:v>Condicionado</x:v>
@@ -2092,13 +2091,13 @@
         <x:v>Restritas</x:v>
       </x:c>
       <x:c r="K37" t="str">
-        <x:v>P</x:v>
+        <x:v>H</x:v>
       </x:c>
       <x:c r="L37" t="str">
         <x:v>https://seer.ufu.br/index.php/revistabrasileiracartografia/about/submissions</x:v>
       </x:c>
       <x:c r="M37" t="str">
-        <x:v>Adota política Elsevier; item obrigatório na submissão.</x:v>
+        <x:v>A RBC declara adotar a política Elsevier e exige confirmar a declaração de IA na submissão. Pela norma adotada, preparação do manuscrito pede seção dedicada e uso metodológico pede Métodos; correções básicas têm dispensas. Imagens explicativas e visualizações de dados têm condições distintas de imagens primárias; não fabricar dados. Revisão: somente apoio humano sob sigilo, ferramentas privadas e declaração conforme a norma geral. Adoção documentada, não inferência pela editora.</x:v>
       </x:c>
       <x:c r="N37" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -2433,10 +2432,10 @@
         <x:v>Restrita</x:v>
       </x:c>
       <x:c r="H45" t="str">
-        <x:v>Seção própria</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I45" t="str">
-        <x:v>Vedado</x:v>
+        <x:v>Não trata</x:v>
       </x:c>
       <x:c r="J45" t="str">
         <x:v>Restritas</x:v>
@@ -2448,7 +2447,7 @@
         <x:v>https://www.asbmb.org/journals/editorial-policies</x:v>
       </x:c>
       <x:c r="M45" t="str">
-        <x:v>Só melhorar texto existente; figuras com IA em regra vedadas.</x:v>
+        <x:v>Nos periódicos ASBMB, IA só pode melhorar texto já existente; código para análise deve ser relatado nos procedimentos experimentais. Redação assistida pede seção dedicada antes das referências; checagens básicas são dispensadas. Figuras são em regra vedadas, salvo método reprodutível ou capa com autorização prévia. A política editorial e a página de revisão consultadas não estabelecem regra específica de GenAI para pareceristas; isso não é permissão.</x:v>
       </x:c>
       <x:c r="N45" t="str">
         <x:v>Ciências Biológicas</x:v>
@@ -2578,7 +2577,7 @@
       <x:c r="L48" t="str">
         <x:v>https://www.cell.com/cell/information-for-authors/journal-policies</x:v>
       </x:c>
-      <x:c r="M48" t="str"/>
+      <x:c r="M48"/>
       <x:c r="N48" t="str">
         <x:v>Ciências Biológicas</x:v>
       </x:c>
@@ -2664,7 +2663,7 @@
       <x:c r="L50" t="str">
         <x:v>https://peerj.com/about/policies-and-procedures/</x:v>
       </x:c>
-      <x:c r="M50" t="str"/>
+      <x:c r="M50"/>
       <x:c r="N50" t="str">
         <x:v>Ciências Biológicas</x:v>
       </x:c>
@@ -3038,9 +3037,7 @@
       <x:c r="E59" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F59" t="n">
-        <x:v>2023</x:v>
-      </x:c>
+      <x:c r="F59"/>
       <x:c r="G59" t="str">
         <x:v>Permitida</x:v>
       </x:c>
@@ -3048,7 +3045,7 @@
         <x:v>Agradecimentos</x:v>
       </x:c>
       <x:c r="I59" t="str">
-        <x:v>Vedado</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J59" t="str">
         <x:v>Não trata</x:v>
@@ -3057,10 +3054,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L59" t="str">
-        <x:v>https://connect.informs.org/discussion/generative-artificial-intelligence-ai-policy-for-reviewers-associate-editors-department-editors-editors-for-informs-journals</x:v>
+        <x:v>https://pubsonline.informs.org/authorportal/publication-ethics</x:v>
       </x:c>
       <x:c r="M59" t="str">
-        <x:v>'Authors are permitted to use generative AI'; declarar em Agradecimentos; revisores e editores vedados.</x:v>
+        <x:v>O portal institucional permite IA sob responsabilidade humana e exige declaração em Agradecimentos com ferramenta e natureza do auxílio. A norma geral de revisão permite apoio somente se o sistema não retiver, compartilhar ou treinar com o conteúdo e cumprir integralmente o sigilo. A proibição citada no fórum de 2023 tratava do IJOC e não deve ser generalizada a todos os títulos; consultar também a regra específica da revista. Fabricação de dados é proibida. A fonte geral não fixa uma regra específica de imagens; ano da versão não explicitado.</x:v>
       </x:c>
       <x:c r="N59" t="str">
         <x:v>Engenharias</x:v>
@@ -3720,7 +3717,7 @@
       <x:c r="L74" t="str">
         <x:v>https://home.liebertpub.com/publications/ai-in-neuroscience/681/for-authors</x:v>
       </x:c>
-      <x:c r="M74" t="str"/>
+      <x:c r="M74"/>
       <x:c r="N74" t="str">
         <x:v>Ciências da Saúde</x:v>
       </x:c>
@@ -3762,7 +3759,7 @@
         <x:v>https://www.scielo.br/journal/csp/about/#instructions</x:v>
       </x:c>
       <x:c r="M75" t="str">
-        <x:v>Só legibilidade/linguagem; sem IA em figuras/tabelas.</x:v>
+        <x:v>Instruções operacionais PT/EN: escrita assistida para legibilidade/linguagem, com controle humano e declaração em Métodos. Figuras, quadros e tabelas não podem ser criados/alterados por IA, salvo quando a IA integra o desenho ou método, descrito de modo reprodutível. A seção operacional de revisão não dá regra específica de GenAI para pareceristas. O editorial 40(11) discute usos mais amplos; não se interpreta essa discussão como dispensa das instruções vigentes.</x:v>
       </x:c>
       <x:c r="N75" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -3790,13 +3787,13 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H76" t="str">
-        <x:v>Seção própria</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I76" t="str">
         <x:v>Não trata</x:v>
       </x:c>
       <x:c r="J76" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Permitidas c/ declaração</x:v>
       </x:c>
       <x:c r="K76" t="str">
         <x:v>P</x:v>
@@ -3805,7 +3802,7 @@
         <x:v>https://www.scielo.br/journal/reben/about/#instructions</x:v>
       </x:c>
       <x:c r="M76" t="str">
-        <x:v>Seção sob Métodos.</x:v>
+        <x:v>Adota recomendações COPE e remete a WAME/JAMA. Deve descrever em Métodos o uso e todos os prompts para texto, adaptações, ilustrações ou tabelas. Para análises, resultados ou código, informar também no Resumo, incluindo prompt completo, ferramenta, versão, data e horário. Referências: IA limitada à normalização. As instruções contemplam ilustrações com declaração, mas isso não autoriza fabricar dados. Não foi localizada nesta página regra própria específica sobre uso de IA por pareceristas.</x:v>
       </x:c>
       <x:c r="N76" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -3970,7 +3967,7 @@
         <x:v>Restrita</x:v>
       </x:c>
       <x:c r="H80" t="str">
-        <x:v>Seção própria</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I80" t="str">
         <x:v>Vedado</x:v>
@@ -3985,7 +3982,7 @@
         <x:v>https://www.sciencesocieties.org/publications/journals/author-resources/editorial-policies</x:v>
       </x:c>
       <x:c r="M80" t="str">
-        <x:v>Só linguagem; nenhum uso por revisores e editores.</x:v>
+        <x:v>Atualizada em 30 de junho de 2026. Na escrita, IA apenas como apoio à legibilidade/linguagem, com controle humano; proíbe criar/alterar dados e resultados originais. Declarar na submissão e em seção própria antes das referências, com ferramenta, versão e validação; ferramentas básicas de gramática, ortografia e referências dispensam. A regra de escrita não regula uso como método de análise. Revisores e editores não podem usar IA generativa na avaliação nem enviar manuscritos a essas ferramentas.</x:v>
       </x:c>
       <x:c r="N80" t="str">
         <x:v>Ciências Agrárias</x:v>
@@ -4094,12 +4091,14 @@
       <x:c r="E83" t="str">
         <x:v>Brasil</x:v>
       </x:c>
-      <x:c r="F83"/>
+      <x:c r="F83" t="n">
+        <x:v>2024</x:v>
+      </x:c>
       <x:c r="G83" t="str">
         <x:v>Restrita</x:v>
       </x:c>
       <x:c r="H83" t="str">
-        <x:v>Seção própria</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I83" t="str">
         <x:v>Não trata</x:v>
@@ -4111,10 +4110,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L83" t="str">
-        <x:v>https://www.scielo.br/journal/rbz/about/?ilang=en</x:v>
+        <x:v>https://rbz.org.br/wp-content/uploads/2024/06/Instructions-to-authors-RBZ-2024.pdf</x:v>
       </x:c>
       <x:c r="M83" t="str">
-        <x:v>Não endossa IA para criar conteúdo.</x:v>
+        <x:v>Diretrizes revisadas em maio de 2024: não endossa criação de conteúdo; admite apoio à linguagem, fluência e organização sob supervisão humana. Declarar na carta e na seção dedicada após Apoio financeiro, indicando natureza/extensão do uso. Nas seções de avaliação e figuras examinadas, não há regra específica de GenAI para pareceristas ou imagens; não inferir autorização.</x:v>
       </x:c>
       <x:c r="N83" t="str">
         <x:v>Ciências Agrárias</x:v>
@@ -4271,22 +4270,22 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H87" t="str">
-        <x:v>Não especifica</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I87" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J87" t="str">
         <x:v>Não trata</x:v>
       </x:c>
       <x:c r="K87" t="str">
-        <x:v>P</x:v>
+        <x:v>H</x:v>
       </x:c>
       <x:c r="L87" t="str">
         <x:v>https://www.scielo.br/journal/rarv/about/?ilang=en</x:v>
       </x:c>
       <x:c r="M87" t="str">
-        <x:v>Adere ao Guia SciELO (que pede Resumo + Métodos), sem regra própria detalhada.</x:v>
+        <x:v>A página do periódico, em PT e EN, adota expressamente o Guia SciELO como boas práticas; não detalha regra própria de IA. O guia preliminar de 14/9/2023 pede relato no Resumo e em Métodos/equivalente e documentação no parecer, com proteção de confidencialidade. Exigências operacionais do título devem ser confirmadas; a herança aqui deriva dessa adoção expressa, não apenas da indexação SciELO. O guia não fixa norma específica para imagens.</x:v>
       </x:c>
       <x:c r="N87" t="str">
         <x:v>Ciências Agrárias</x:v>
@@ -4316,7 +4315,7 @@
         <x:v>Restrita</x:v>
       </x:c>
       <x:c r="H88" t="str">
-        <x:v>Seção própria</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I88" t="str">
         <x:v>Não trata</x:v>
@@ -4331,7 +4330,7 @@
         <x:v>https://www.scielo.br/journal/cr/about/</x:v>
       </x:c>
       <x:c r="M88" t="str">
-        <x:v>Sem IA para escrever, resumo, palavras-chave, hipóteses ou conclusão; revisão de redação e melhoria de imagens com declaração; IA como método em M&amp;M.</x:v>
+        <x:v>Não admite IA para redigir o manuscrito, resumo, palavras-chave, hipóteses ou conclusão. Permite revisão linguística e melhoria de imagens sem inserir/remover elementos que alterem a interpretação, sob supervisão e declaração em seção adequada. IA integrada à metodologia deve ser descrita reprodutivelmente em Materiais e Métodos. A página não fixa título único da declaração nem regra própria de pareceristas.</x:v>
       </x:c>
       <x:c r="N88" t="str">
         <x:v>Ciências Agrárias</x:v>
@@ -4463,7 +4462,7 @@
       <x:c r="L91" t="str">
         <x:v>https://www.aeaweb.org/journals/aer/editorial-policy</x:v>
       </x:c>
-      <x:c r="M91" t="str"/>
+      <x:c r="M91"/>
       <x:c r="N91" t="str">
         <x:v>Ciências Sociais Aplicadas</x:v>
       </x:c>
@@ -4548,7 +4547,7 @@
         <x:v>https://www.aom.org/publications/journals/publishing-with-aom/aom-artificial-intelligence-policy</x:v>
       </x:c>
       <x:c r="M93" t="str">
-        <x:v>Declarar uso em cada etapa.</x:v>
+        <x:v>Autores podem usar IA sob responsabilidade humana e devem informar seu uso em cada etapa, confirmar verificação dos resultados e fornecer detalhes se solicitados. Para periódicos, informar modelo e finalidade na carta de apresentação e nos agradecimentos; para o encontro anual, na folha de rosto. Pareceristas podem melhorar a clareza do próprio texto, mas não gerar pareceres nem enviar manuscritos, figuras ou dados à IA; editores também preservam sigilo dos pareceres. A etapa de apresentação inclui figuras, mas não há aqui política específica separada de imagens.</x:v>
       </x:c>
       <x:c r="N93" t="str">
         <x:v>Ciências Sociais Aplicadas</x:v>
@@ -4581,7 +4580,7 @@
         <x:v>Não especifica</x:v>
       </x:c>
       <x:c r="I94" t="str">
-        <x:v>Condicionado</x:v>
+        <x:v>Não trata</x:v>
       </x:c>
       <x:c r="J94" t="str">
         <x:v>Não trata</x:v>
@@ -4593,7 +4592,7 @@
         <x:v>https://www.natcom.org/wp-content/uploads/2026/02/Guidance-on-AI-Use-for-Submitters.pdf</x:v>
       </x:c>
       <x:c r="M94" t="str">
-        <x:v>Política associativa em votação (nov/2026).</x:v>
+        <x:v>Orientação para submissões à convenção NCA, vigente no ciclo 2026; não é uma política universal de todos os periódicos da associação. Recomenda transparência sobre usos substanciais e consulta às exigências da unidade/divisão; correções menores geralmente dispensam declaração. Autores respondem por originalidade, fatos e referências, e não devem inserir dados confidenciais ou pessoais em plataformas públicas. Não especifica seção única nem regra própria de pareceristas ou imagens; menciona visualizações entre usos a declarar.</x:v>
       </x:c>
       <x:c r="N94" t="str">
         <x:v>Ciências Sociais Aplicadas</x:v>
@@ -4635,7 +4634,7 @@
       <x:c r="L95" t="str">
         <x:v>https://www.aals.org/</x:v>
       </x:c>
-      <x:c r="M95" t="str"/>
+      <x:c r="M95"/>
       <x:c r="N95" t="str">
         <x:v>Ciências Sociais Aplicadas</x:v>
       </x:c>
@@ -4745,29 +4744,27 @@
       <x:c r="E98" t="str">
         <x:v>Reino Unido</x:v>
       </x:c>
-      <x:c r="F98" t="n">
-        <x:v>2024</x:v>
-      </x:c>
+      <x:c r="F98"/>
       <x:c r="G98" t="str">
-        <x:v>Restrita</x:v>
+        <x:v>Vedada</x:v>
       </x:c>
       <x:c r="H98" t="str">
-        <x:v>Não especifica</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I98" t="str">
         <x:v>Não trata</x:v>
       </x:c>
       <x:c r="J98" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Restritas</x:v>
       </x:c>
       <x:c r="K98" t="str">
         <x:v>P</x:v>
       </x:c>
       <x:c r="L98" t="str">
-        <x:v>https://elgar.blog/2024/11/19/academic-writing-in-the-age-of-ai-benefits-risks-and-ethics</x:v>
+        <x:v>https://www.e-elgar.com/author-hub/as-you-write-your-book-or-chapter/</x:v>
       </x:c>
       <x:c r="M98" t="str">
-        <x:v>Conteúdo substantivo gerado por IA não permitido.</x:v>
+        <x:v>Norma para livros/capítulos: não permite redigir, reescrever ou parafrasear texto com GenAI; admite verificadores linguísticos limitados. Uso além de apoio menor deve ser declarado na proposta, checklist e manuscrito quando exigido. Não incluir imagens geradas sem discutir previamente com o editor; vedado fabricar/manipular dados ou imagens originais. A página não estabelece regra específica de IA para pareceristas. Sem data normativa explícita.</x:v>
       </x:c>
       <x:c r="N98" t="str">
         <x:v>Ciências Sociais Aplicadas</x:v>
@@ -4921,18 +4918,20 @@
       <x:c r="E102" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F102"/>
+      <x:c r="F102" t="n">
+        <x:v>2025</x:v>
+      </x:c>
       <x:c r="G102" t="str">
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H102" t="str">
-        <x:v>Métodos</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I102" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J102" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Permitidas c/ declaração</x:v>
       </x:c>
       <x:c r="K102" t="str">
         <x:v>P</x:v>
@@ -4941,7 +4940,7 @@
         <x:v>https://www.apa.org/pubs/journals/resources/publishing-tips/policy-generative-ai</x:v>
       </x:c>
       <x:c r="M102" t="str">
-        <x:v>Declarar em Métodos e citar.</x:v>
+        <x:v>Página criada em novembro de 2023 e atualizada em agosto de 2025. A regra geral pede declaração e citação em Métodos; a orientação detalhada distingue Introdução, Métodos, nota do autor ou seção da figura conforme o uso, sujeita às exigências do editor. Autores verificam informação e referências e preservam registros e prompts. Editores e pareceristas não podem inserir materiais submetidos em IA generativa por confidencialidade. A orientação contempla criação/edição de figuras com declaração, sem dispensar validação ou autorizar fabricação de dados.</x:v>
       </x:c>
       <x:c r="N102" t="str">
         <x:v>Ciências Humanas</x:v>
@@ -4983,7 +4982,7 @@
       <x:c r="L103" t="str">
         <x:v>https://www.aera.net/</x:v>
       </x:c>
-      <x:c r="M103" t="str"/>
+      <x:c r="M103"/>
       <x:c r="N103" t="str">
         <x:v>Ciências Humanas</x:v>
       </x:c>
@@ -5027,7 +5026,7 @@
         <x:v>https://www.aag.org/statement-of-professional-ethics/</x:v>
       </x:c>
       <x:c r="M104" t="str">
-        <x:v>Código de ética profissional.</x:v>
+        <x:v>Código de ética profissional: geógrafos devem reconhecer, documentar cuidadosamente e justificar como e por que utilizaram IA em pesquisa, ensino, propostas e correspondência. A regra não determina seção única para manuscritos, nem instruções específicas de IA por pareceristas ou para imagens sintéticas. Responsabilidade, privacidade e confidencialidade da pesquisa continuam obrigatórias; consultar a revista para exigências editoriais adicionais.</x:v>
       </x:c>
       <x:c r="N104" t="str">
         <x:v>Ciências Humanas</x:v>
@@ -5159,7 +5158,7 @@
       <x:c r="L107" t="str">
         <x:v>https://www.asanet.org/about/asa-code-of-ethics/</x:v>
       </x:c>
-      <x:c r="M107" t="str"/>
+      <x:c r="M107"/>
       <x:c r="N107" t="str">
         <x:v>Ciências Humanas</x:v>
       </x:c>
@@ -5203,7 +5202,7 @@
         <x:v>https://ajps.org/ajps-ai-policy/</x:v>
       </x:c>
       <x:c r="M108" t="str">
-        <x:v>Não declarar = motivo de recusa.</x:v>
+        <x:v>Política do American Journal of Political Science, periódico da Midwest Political Science Association publicado pela Wiley; não é regra geral da APSA. Atualização de 11 de agosto de 2026. Declaração consolidada em nota de rodapé deve refletir o questionário de submissão, identificar ferramenta, tarefa e supervisão; usos mínimos não generativos são dispensados. Falha em declarar pode motivar recusa. Pareceristas não enviam manuscritos à IA, mas podem organizar ideias e melhorar o próprio texto sem conteúdo confidencial e devem declarar apoio à redação. Imagens figuram nos usos a declarar, sem regra específica de permissão nesta página.</x:v>
       </x:c>
       <x:c r="N108" t="str">
         <x:v>Ciências Humanas</x:v>
@@ -5245,7 +5244,7 @@
       <x:c r="L109" t="str">
         <x:v>https://www.apaonline.org/</x:v>
       </x:c>
-      <x:c r="M109" t="str"/>
+      <x:c r="M109"/>
       <x:c r="N109" t="str">
         <x:v>Ciências Humanas</x:v>
       </x:c>
@@ -5286,7 +5285,7 @@
       <x:c r="L110" t="str">
         <x:v>https://papers.aarweb.org/units</x:v>
       </x:c>
-      <x:c r="M110" t="str"/>
+      <x:c r="M110"/>
       <x:c r="N110" t="str">
         <x:v>Ciências Humanas</x:v>
       </x:c>
@@ -5370,10 +5369,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L112" t="str">
-        <x:v>https://utpress.utexas.edu/generative-ai-policy-for-authors</x:v>
+        <x:v>https://utpress.utexas.edu/generative-ai-policy-for-authors/</x:v>
       </x:c>
       <x:c r="M112" t="str">
-        <x:v>Limite de 5% de texto gerado.</x:v>
+        <x:v>Política de maio de 2025: não aceita obra com 5% ou mais da contagem total de palavras escritos/gerados por IA. Autores devem informar o editor ao concordar com a submissão para revisão e incluir declaração no início da obra, descrevendo usos em texto, imagens, gráficos e tabelas; cada uso deve ser citado. Imagens geradas exigem aprovação prévia da Press. Revistas individuais podem ter diretrizes próprias. A página não estabelece regra de uso de IA por pareceristas.</x:v>
       </x:c>
       <x:c r="N112" t="str">
         <x:v>Ciências Humanas</x:v>
@@ -5589,10 +5588,10 @@
         <x:v>H</x:v>
       </x:c>
       <x:c r="L117" t="str">
-        <x:v>https://prc.springeropen.com/</x:v>
+        <x:v>https://link.springer.com/journal/41155/submission-guidelines</x:v>
       </x:c>
       <x:c r="M117" t="str">
-        <x:v>Descontinuada da coleção SciELO (out/2026); publicada pela SpringerOpen — política Springer Nature herdada; cláusula própria não localizada.</x:v>
+        <x:v>O link de políticas editoriais do próprio periódico encaminha às políticas Springer, cuja seção de IA estabelece avaliação por risco para autores, revisores e editores. Apoio assistivo é permitido; uso interpretativo exige supervisão, verificação e transparência. Não se pode delegar julgamento, fabricar dados ou criar deepfakes fotorealistas. Revisores não enviam conteúdo a IA pública/insegura. Não há seção universal de declaração nem data normativa explícita. A herança foi conferida no encaminhamento do título; consultar suas instruções próprias.</x:v>
       </x:c>
       <x:c r="N117" t="str">
         <x:v>Ciências Humanas</x:v>
@@ -5636,7 +5635,7 @@
       <x:c r="L118" t="str">
         <x:v>https://www.mla.org/Publications/MLA-Book-Publications/Resources-for-Contributors/Policy-on-Generative-AI</x:v>
       </x:c>
-      <x:c r="M118" t="str"/>
+      <x:c r="M118"/>
       <x:c r="N118" t="str">
         <x:v>Linguística, Letras e Artes</x:v>
       </x:c>
@@ -5666,7 +5665,7 @@
         <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I119" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Vedado</x:v>
       </x:c>
       <x:c r="J119" t="str">
         <x:v>Permitidas c/ declaração</x:v>
@@ -5677,7 +5676,9 @@
       <x:c r="L119" t="str">
         <x:v>https://www.cambridge.org/core/journals/proceedings-of-the-linguistic-society-of-america/information/author-instructions/preparing-your-materials</x:v>
       </x:c>
-      <x:c r="M119" t="str"/>
+      <x:c r="M119" t="str">
+        <x:v>Norma do Proceedings of the Linguistic Society of America, não de todas as publicações da LSA. Declarar texto/tradução em Agradecimentos ou nota, dados em Métodos e imagens nas legendas, com ferramenta, versão, datas e descrição; usos mínimos não generativos dispensam. Pareceres devem resultar da escrita e do julgamento do revisor; apoio limitado a correção mínima não generativa. Manuscrito e parecer não podem ser compartilhados com IA; a própria página pede consulta prévia ao editor sobre compartilhamento.</x:v>
+      </x:c>
       <x:c r="N119" t="str">
         <x:v>Linguística, Letras e Artes</x:v>
       </x:c>
@@ -5718,7 +5719,7 @@
       <x:c r="L120" t="str">
         <x:v>https://www.collegeart.org/</x:v>
       </x:c>
-      <x:c r="M120" t="str"/>
+      <x:c r="M120"/>
       <x:c r="N120" t="str">
         <x:v>Linguística, Letras e Artes</x:v>
       </x:c>
@@ -5757,10 +5758,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L121" t="str">
-        <x:v>https://www.scielo.br/journal/delta/about/#instructions</x:v>
+        <x:v>https://revistas.pucsp.br/delta/about/submissions</x:v>
       </x:c>
       <x:c r="M121" t="str">
-        <x:v>IA pode apoiar revisores em checagens técnicas.</x:v>
+        <x:v>Política própria nas normas de submissão: autores devem garantir originalidade e contribuição e explicitar a extensão do envolvimento de IA. Geração, análise ou qualquer outro uso devem ser informados em Materiais e Métodos. Na revisão, IA pode apoiar identificação de plágio, inconsistências e aspectos técnicos, sem substituir a decisão humana. Dados pessoais devem obedecer diretrizes de privacidade e anonimização. Não estabelece regra específica de imagens nem data normativa explícita.</x:v>
       </x:c>
       <x:c r="N121" t="str">
         <x:v>Linguística, Letras e Artes</x:v>
@@ -5959,9 +5960,7 @@
       <x:c r="E126" t="str">
         <x:v>Internacional</x:v>
       </x:c>
-      <x:c r="F126" t="n">
-        <x:v>2025</x:v>
-      </x:c>
+      <x:c r="F126"/>
       <x:c r="G126" t="str">
         <x:v>Permitida</x:v>
       </x:c>
@@ -5978,9 +5977,11 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L126" t="str">
-        <x:v>https://www.wiley.com/en-us/publishing/article/ai-guidelines</x:v>
-      </x:c>
-      <x:c r="M126" t="str"/>
+        <x:v>https://authors.wiley.com/ethics-guidelines/index.html</x:v>
+      </x:c>
+      <x:c r="M126" t="str">
+        <x:v>Uso responsável como apoio, não substituto do julgamento humano. Uso substancial, desenvolvimento ou tradução devem ser declarados na submissão e integrados ao manuscrito; correção ortográfica, gramatical e edição geral são dispensadas. Ilustrações e visualizações são possíveis, com restrições para fotografias; confirmar detalhes e regra do título. Pareceristas podem apenas melhorar clareza/linguagem do próprio parecer, declarando ao editor, sem enviar manuscrito, figuras ou tabelas nem delegar a avaliação.</x:v>
+      </x:c>
       <x:c r="N126" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6109,7 +6110,9 @@
       <x:c r="L129" t="str">
         <x:v>https://academic.oup.com/pages/for-authors/journals/preparing-and-submitting-your-manuscript/ai-principles-for-oxford-journals</x:v>
       </x:c>
-      <x:c r="M129" t="str"/>
+      <x:c r="M129" t="str">
+        <x:v>Política para autores atualizada em 13 de julho de 2026; requisitos próprios do periódico prevalecem. Usos substanciais, tradução, código e visualização geralmente exigem declaração na carta e nos Agradecimentos, também em Métodos quando integrarem o método, com ferramenta, versão, finalidade e supervisão. Correção linguística simples e formatação de referências dispensam. Ilustrações e resumos gráficos podem ser admitidos com declaração; é proibido fabricar resultados ou criar/alterar imagens científicas factuais. Os princípios gerais exigem responsabilidade e confidencialidade de autores, revisores e editores; verificar instruções específicas de revisão do título.</x:v>
+      </x:c>
       <x:c r="N129" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6150,7 +6153,9 @@
       <x:c r="L130" t="str">
         <x:v>https://www.cambridge.org/core/services/publishing-ethics/authorship-and-contributorship-journals</x:v>
       </x:c>
-      <x:c r="M130" t="str"/>
+      <x:c r="M130" t="str">
+        <x:v>Autores devem declarar e explicar o uso de IA, não a listar como autora, assegurar integridade, atribuição e originalidade e observar exigências adicionais do periódico. A página geral não fixa seção universal de declaração nem regra específica para imagens. Na revisão, compartilhar manuscritos ou propostas com LLMs constitui quebra de confidencialidade e má conduta; políticas próprias dos títulos podem ser mais restritivas.</x:v>
+      </x:c>
       <x:c r="N130" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6193,7 +6198,7 @@
       <x:c r="L131" t="str">
         <x:v>https://www.degruyterbrill.com/publishing/for-authors/author-policies/artificial-intelligence</x:v>
       </x:c>
-      <x:c r="M131" t="str"/>
+      <x:c r="M131"/>
       <x:c r="N131" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6263,21 +6268,23 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H133" t="str">
-        <x:v>Não especifica</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I133" t="str">
         <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J133" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Permitidas c/ declaração</x:v>
       </x:c>
       <x:c r="K133" t="str">
         <x:v>P</x:v>
       </x:c>
       <x:c r="L133" t="str">
-        <x:v>https://www.frontiersin.org/about/policies-and-publication-ethics</x:v>
-      </x:c>
-      <x:c r="M133" t="str"/>
+        <x:v>https://www.frontiersin.org/guidelines/policies-and-publication-ethics</x:v>
+      </x:c>
+      <x:c r="M133" t="str">
+        <x:v>Texto gerado deve ser declarado em Agradecimentos; conteúdo textual ou visual produzido/editado com IA também em Métodos quando pertinente, com ferramenta, versão, modelo e fonte. Figuras são admitidas sob verificação de fidelidade aos dados e ausência de plágio; recomenda preservar prompts e saídas em suplementos. Manuscritos não podem ser enviados a ferramentas externas. Pareceristas dispõem de apoio interno seguro, sem delegar decisão editorial; eventual uso externo exige discussão e aprovação prévia e divulgação aos autores.</x:v>
+      </x:c>
       <x:c r="N133" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6318,7 +6325,9 @@
       <x:c r="L134" t="str">
         <x:v>https://journals.plos.org/plosone/s/ethical-publishing-practice</x:v>
       </x:c>
-      <x:c r="M134" t="str"/>
+      <x:c r="M134" t="str">
+        <x:v>Permite apoio à pesquisa e à redação, com responsabilidade humana e sem fabricação de dados. Declarar ferramenta, finalidade, partes afetadas e validação em Métodos, Agradecimentos ou legenda pertinente. Correção/reformulação linguística e carta de apresentação dispensam declaração; tradução é recomendada, não obrigatória. Pareceristas e editores não enviam submissões nem resumos confidenciais à IA e não a usam para resumir ou avaliar o manuscrito; apoio geral ou linguístico sem conteúdo confidencial é possível e deve ser declarado no parecer/decisão. Imagens ilustrativas são admitidas com legenda e validação, sem deturpar resultados primários.</x:v>
+      </x:c>
       <x:c r="N134" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6359,7 +6368,7 @@
       <x:c r="L135" t="str">
         <x:v>https://f1000research.com/about/policies</x:v>
       </x:c>
-      <x:c r="M135" t="str"/>
+      <x:c r="M135"/>
       <x:c r="N135" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6400,7 +6409,7 @@
       <x:c r="L136" t="str">
         <x:v>https://www.science.org/content/page/science-journals-editorial-policies</x:v>
       </x:c>
-      <x:c r="M136" t="str"/>
+      <x:c r="M136"/>
       <x:c r="N136" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6528,7 +6537,7 @@
         <x:v>https://www.scielo.br/journal/aabc/about/#instructions</x:v>
       </x:c>
       <x:c r="M139" t="str">
-        <x:v>Seção de IA declara a política 'em estudo' (16/10/2026).</x:v>
+        <x:v>Na seção específica de IA, consultada em PT e EN em 17 de outubro de 2026, o periódico informa que está estudando quais usos/contextos serão permitidos para atualizar sua política editorial. Esta informação não autoriza irrestritamente a geração de conteúdo e não especifica local de declaração, uso por pareceristas ou imagens. A codificação de ausência limita-se à política publicada examinada.</x:v>
       </x:c>
       <x:c r="N139" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -6707,10 +6716,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L143" t="str">
-        <x:v>https://grants.nih.gov/grants/guide/notice-files/NOT-OD-25-132.html</x:v>
+        <x:v>https://www.grants.nih.gov/grants/guide/notice-files/NOT-OD-25-132.html</x:v>
       </x:c>
       <x:c r="M143" t="str">
-        <x:v>Proposta substancialmente gerada por IA não é original; 6 propostas/ano.</x:v>
+        <x:v>NOT-OD-25-132, de 17/7/2025, vigente para submissões a partir de 25/9/2025: propostas ou seções substancialmente desenvolvidas por IA não são consideradas ideias originais dos proponentes; apoio limitado pode ser apropriado, sem limiar percentual definido. Não é norma de redação de artigos. NOT-OD-23-149, de 23/6/2023, proíbe IA generativa para analisar/formular pareceres de propostas; exceções de acessibilidade exigem consulta prévia ao responsável federal. Não fixa local de declaração autoral nem política específica de imagens nessas fontes.</x:v>
       </x:c>
       <x:c r="N143" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -6871,7 +6880,7 @@
         <x:v>Alemanha</x:v>
       </x:c>
       <x:c r="F147" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="G147" t="str">
         <x:v>N/A</x:v>
@@ -6889,10 +6898,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L147" t="str">
-        <x:v>https://www.ufz.de/export/data/2/308041_de_K%C3%BCnstliche%20Intelligenz%20in%20der%20wissenschaftlichen%20Begutachtung.%20Position%20und%20Perspektiven%20der%20DFG.pdf</x:v>
+        <x:v>https://www.dfg.de/resource/blob/393362/forschung-2026-01.pdf</x:v>
       </x:c>
       <x:c r="M147" t="str">
-        <x:v>Pareceristas: só sistemas seguros.</x:v>
+        <x:v>Diretriz aprovada em dezembro de 2025, publicada/liberada em 2026. Na avaliação de propostas, IA só apoia o trabalho: julgamento e recomendação permanecem humanos. Exige anuência dos envolvidos, confidencialidade e sistemas locais, institucionais ou nuvem com garantias contratuais e configurações que impeçam retenção/treinamento indevidos. Declarar finalidade e extensão do apoio à DFG; correção técnica sem efeito científico dispensa. Responsabilidade e validação do parecer são pessoais. O registro não classifica redação autoral de artigos nem política específica de imagens.</x:v>
       </x:c>
       <x:c r="N147" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -6969,10 +6978,10 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H149" t="str">
-        <x:v>Não especifica</x:v>
+        <x:v>Submissão/carta</x:v>
       </x:c>
       <x:c r="I149" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J149" t="str">
         <x:v>Não trata</x:v>
@@ -6983,7 +6992,9 @@
       <x:c r="L149" t="str">
         <x:v>https://wennergren.org/ai-policy/</x:v>
       </x:c>
-      <x:c r="M149" t="str"/>
+      <x:c r="M149" t="str">
+        <x:v>Política de 19/03/2025. Proponentes são fortemente encorajados a declarar uso em seção confidencial da proposta, invisível aos revisores, com ferramentas, prompts e verificação; não é obrigação geral. Revisores não podem enviar propostas, rascunhos de parecer, notas ou avaliações a GenAI, mesmo com promessa de não treinamento, nem tentar detectar uso pelo proponente. Sem regra específica para imagens nesta página.</x:v>
+      </x:c>
       <x:c r="N149" t="str">
         <x:v>Ciências Humanas</x:v>
       </x:c>
@@ -7021,7 +7032,7 @@
       <x:c r="K150" t="str">
         <x:v>NL</x:v>
       </x:c>
-      <x:c r="L150" t="str"/>
+      <x:c r="L150"/>
       <x:c r="M150" t="str">
         <x:v>Nenhuma norma específica localizada.</x:v>
       </x:c>
@@ -7107,10 +7118,8 @@
           <x:t xml:space="preserve">Verificação</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P = política lida em fonte primária; S = fonte secundária; H = política herdada da editora (instrução do periódico não lida); A = ausência de regra verificada na fonte primária; NL = não localizado na busca</x:t>
-        </x:is>
+      <x:c r="B6" s="3" t="str">
+        <x:v>P = fonte primária; S = fonte secundária; H = regra herdada com adoção aplicável documentada nos registros reconfirmados; A = ausência no escopo examinado; NL = não localizado. Códigos históricos dos pendentes não certificam releitura atual; consultar o histórico.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -7125,14 +7134,14 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Data de referência</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="3" t="str">
-        <x:v>Base histórica: 16/10/2026; revisão parcial em 17/10/2026: 58/149 registros reconciliados, 40 corrigidos, 91 pendentes. Data de revisão integral não avançou. Histórico: https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-17.json</x:v>
+      <x:c r="B8" s="4" t="str">
+        <x:v>Base histórica: 16/10/2026; revisão parcial em 17/10/2026: 97/149 registros reconciliados, 77 corrigidos, 52 pendentes. Data de revisão integral não avançou. Histórico: https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-17.json</x:v>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>

<commit_message>
Verify official WAME AMS ACM MDPI and De Gruyter policies
</commit_message>
<xml_diff>
--- a/public/levantamentos/politicas-ia/base-politicas-ia-2026-10.xlsx
+++ b/public/levantamentos/politicas-ia/base-politicas-ia-2026-10.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="1" r:id="Re7101c99ab2c4398"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livro de códigos" sheetId="2" r:id="Ra2cef9c784da49b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="1" r:id="R377184d361d44d3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livro de códigos" sheetId="2" r:id="Ra44993badead4783"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -627,16 +627,16 @@
         <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J4" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Permitidas c/ declaração</x:v>
       </x:c>
       <x:c r="K4" t="str">
         <x:v>P</x:v>
       </x:c>
       <x:c r="L4" t="str">
-        <x:v>https://wame.org/page3.php?id=110</x:v>
+        <x:v>https://wame.org/page3.php?id=106</x:v>
       </x:c>
       <x:c r="M4" t="str">
-        <x:v>Ferramenta, versão, data e prompts quando IA afeta análise/código.</x:v>
+        <x:v>Versão 2, 31/05/2023. Texto novo: Agradecimentos e prompts, inclusive conversão para tabelas/ilustrações. Análise, resultados, figuras ou código: Resumo e Métodos, ferramenta/versão, prompt e data/hora. Autores respondem pela integridade e não podem fabricar dados. Editores e pareceristas devem explicar o uso; enviar manuscrito a chatbot viola sigilo. Isso não é autorização geral para qualquer imagem sintética.</x:v>
       </x:c>
       <x:c r="N4" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -1017,9 +1017,7 @@
       <x:c r="E13" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F13" t="n">
-        <x:v>2023</x:v>
-      </x:c>
+      <x:c r="F13"/>
       <x:c r="G13" t="str">
         <x:v>Permitida</x:v>
       </x:c>
@@ -1027,19 +1025,19 @@
         <x:v>Métodos</x:v>
       </x:c>
       <x:c r="I13" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J13" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Permitidas c/ declaração</x:v>
       </x:c>
       <x:c r="K13" t="str">
         <x:v>P</x:v>
       </x:c>
       <x:c r="L13" t="str">
-        <x:v>https://ams.org/publications/journals/policies/UseofArtificialIntelligence</x:v>
+        <x:v>https://www.ams.org/publications/journals/policies/UseofArtificialIntelligence</x:v>
       </x:c>
       <x:c r="M13" t="str">
-        <x:v>Reproduz o COPE.</x:v>
+        <x:v>Adapta posição COPE de fevereiro de 2023, sem data explícita da adoção AMS. Uso na escrita, imagens/elementos gráficos e dados deve ser relatado em Métodos ou equivalente, com ferramenta e finalidade. Responsabilidade humana. Editores e revisores não podem enviar o artigo a LLM em formato algum e por motivo algum; não se infere vedação de todo apoio não confidencial.</x:v>
       </x:c>
       <x:c r="N13" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -1264,7 +1262,7 @@
         <x:v>https://www.acm.org/publications/policies/new-acm-policy-on-authorship</x:v>
       </x:c>
       <x:c r="M18" t="str">
-        <x:v>Uso na pesquisa em Métodos; redação sem declaração geral.</x:v>
+        <x:v>Autoria atualizada em 14/05/2026: não exige declaração de IA para escrita; usos que afetam desenho, método, dados, código e figuras relevantes às conclusões devem ser detalhados em Métodos. Autores humanos respondem pela integridade. Revisão (30/11/2023): só aprimorar qualidade/legibilidade do próprio parecer, removendo toda informação confidencial ou identificadora; não delegar autoria/julgamento. A norma não dá autorização genérica para qualquer imagem sintética.</x:v>
       </x:c>
       <x:c r="N18" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -2008,10 +2006,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L35" t="str">
-        <x:v>https://www.mdpi.com/ethics</x:v>
+        <x:v>https://www.mdpi.com/journal/remotesensing/instructions</x:v>
       </x:c>
       <x:c r="M35" t="str">
-        <x:v>Submissão + Métodos + Agradecimentos.</x:v>
+        <x:v>Instruções do Remote Sensing exigem detalhar uso substantivo em Métodos e identificar ferramenta/finalidade nos Agradecimentos; edição superficial é dispensada. O título adota expressamente a ética MDPI: declaração também na submissão, integridade de dados/imagens, apoio linguístico limitado ao próprio parecer com declaração e sem upload do material, e vedação de GenAI na decisão por editores acadêmicos.</x:v>
       </x:c>
       <x:c r="N35" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -6184,7 +6182,7 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H131" t="str">
-        <x:v>Não especifica</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I131" t="str">
         <x:v>Condicionado</x:v>
@@ -6198,7 +6196,9 @@
       <x:c r="L131" t="str">
         <x:v>https://www.degruyterbrill.com/publishing/for-authors/author-policies/artificial-intelligence</x:v>
       </x:c>
-      <x:c r="M131"/>
+      <x:c r="M131" t="str">
+        <x:v>Setembro de 2026: não aceita trabalhos gerados por IA; autores humanos respondem pelo conteúdo. Contribuição substantiva de IA deve ser declarada; método/desenho: Agradecimentos; proofreading/copy-editing simples são dispensados. Admite ilustrações e capas legais, declaradas na submissão; proíbe fabricar/alterar dados, figuras e imagens experimentais. Revisores não podem enviar manuscrito ou partes a IA; avaliação é responsabilidade exclusivamente humana.</x:v>
+      </x:c>
       <x:c r="N131" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6240,7 +6240,7 @@
         <x:v>https://www.mdpi.com/ethics</x:v>
       </x:c>
       <x:c r="M132" t="str">
-        <x:v>Editores acadêmicos proibidos de usar IA.</x:v>
+        <x:v>GenAI substantiva deve ser declarada na submissão, detalhada em Materiais e Métodos e identificada nos Agradecimentos. Edição gramatical, estrutural, ortográfica e formatação são dispensadas. Admite gráficos/conteúdo gerado sob integridade e responsabilidade humana, sem fabricar ou manipular dados/imagens originais. Pareceristas: apoio limitado à qualidade da escrita, declarado; nunca upload de manuscrito, figuras, tabelas ou comunicações. Editores acadêmicos não podem usar GenAI na revisão ou decisão editorial.</x:v>
       </x:c>
       <x:c r="N132" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -7141,7 +7141,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="4" t="str">
-        <x:v>Base histórica: 16/10/2026; revisão parcial em 17/10/2026: 97/149 registros reconciliados, 77 corrigidos, 52 pendentes. Data de revisão integral não avançou. Histórico: https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-17.json</x:v>
+        <x:v>Base histórica: 16/10/2026; revisão parcial em 17/10/2026: 103/149 registros reconciliados, 83 corrigidos, 46 pendentes. Data de revisão integral não avançou. Histórico: https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-17.json</x:v>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>

<commit_message>
Clarify conditional permissions without implying universal disclosure
</commit_message>
<xml_diff>
--- a/public/levantamentos/politicas-ia/base-politicas-ia-2026-10.xlsx
+++ b/public/levantamentos/politicas-ia/base-politicas-ia-2026-10.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="1" r:id="R377184d361d44d3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livro de códigos" sheetId="2" r:id="Ra44993badead4783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="1" r:id="R274ceb5590ad41a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livro de códigos" sheetId="2" r:id="Ra0a6368d6ddc4c16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7072,10 +7072,8 @@
           <x:t xml:space="preserve">Geração de texto pelo autor</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Permitida = usos substantivos admitidos com declaração; Restrita = só edição/linguagem ou apoio auxiliar; Vedada = proíbe gerar conteúdo/texto com IA; Sem regra = nada localizado; N/A = não se aplica</x:t>
-        </x:is>
+      <x:c r="B2" s="3" t="str">
+        <x:v>Permitida = usos substantivos admitidos sob condições; declaração depende da regra. Restrita = só edição/apoio; Vedada = proíbe gerar texto; Sem regra = nada localizado no escopo; N/A = não se aplica.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">

</xml_diff>

<commit_message>
Reconcile EMBO Press and ASAS policies with official guidance
</commit_message>
<xml_diff>
--- a/public/levantamentos/politicas-ia/base-politicas-ia-2026-10.xlsx
+++ b/public/levantamentos/politicas-ia/base-politicas-ia-2026-10.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="1" r:id="R274ceb5590ad41a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livro de códigos" sheetId="2" r:id="Ra0a6368d6ddc4c16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="1" r:id="R66e10773eb1949a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livro de códigos" sheetId="2" r:id="Rb0051a8e674b4e75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2399,10 +2399,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L44" t="str">
-        <x:v>https://www.embopress.org/page/journal/14602075/authorguide</x:v>
+        <x:v>https://link.springer.com/partners/embo-press/editorial-policies</x:v>
       </x:c>
       <x:c r="M44" t="str">
-        <x:v>Uso 'primarily restricted' a estilo e qualidade; declaração no artigo publicado.</x:v>
+        <x:v>Uso principalmente restrito a melhorar estilo, acessibilidade e qualidade do texto e das imagens humanos, com verificação e responsabilidade dos autores. Declarar no artigo as partes assistidas e as ferramentas, sem seção geral fixa. Uso em coleta/análise deve constar em Métodos; dados sintéticos exigem identificação no texto, figura e Métodos, sem falsificar evidência experimental. Ilustração e visualização podem ser admitidas com declaração e atribuição. As seções de revisão consultadas exigem sigilo, mas não estabelecem disposição específica sobre IA; Não trata não significa autorização.</x:v>
       </x:c>
       <x:c r="N44" t="str">
         <x:v>Ciências Biológicas</x:v>
@@ -4054,19 +4054,19 @@
         <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I82" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J82" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Permitidas c/ declaração</x:v>
       </x:c>
       <x:c r="K82" t="str">
         <x:v>P</x:v>
       </x:c>
       <x:c r="L82" t="str">
-        <x:v>https://academic.oup.com/jas/pages/General_Instructions</x:v>
+        <x:v>https://academic.oup.com/jas/pages/author-guidelines</x:v>
       </x:c>
       <x:c r="M82" t="str">
-        <x:v>Carta + Métodos/Agradecimentos.</x:v>
+        <x:v>Regra própria do Journal of Animal Science: declarar uso de IA para conteúdo, imagens, código, dados ou tradução tanto na carta quanto em Métodos ou Agradecimentos; IA não é autora. Imagens assistidas exigem declaração e não podem falsificar dados. Os princípios gerais OUP aplicam responsabilidade e proteção do sigilo a revisores e editores; uso condicionado não autoriza delegar julgamento científico nem expor manuscritos a serviços externos. As exigências específicas do periódico prevalecem sobre a orientação geral para autores.</x:v>
       </x:c>
       <x:c r="N82" t="str">
         <x:v>Ciências Agrárias</x:v>
@@ -7139,7 +7139,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="4" t="str">
-        <x:v>Base histórica: 16/10/2026; revisão parcial em 17/10/2026: 103/149 registros reconciliados, 83 corrigidos, 46 pendentes. Data de revisão integral não avançou. Histórico: https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-17.json</x:v>
+        <x:v>Base histórica: 16/10/2026; revisão parcial em 17/10/2026: 105/149 registros reconciliados, 85 corrigidos, 44 pendentes. Data de revisão integral não avançou. Histórico: https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-17.json</x:v>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>

<commit_message>
Conclui reconciliacao das 149 politicas com fontes e exports consistentes
</commit_message>
<xml_diff>
--- a/public/levantamentos/politicas-ia/base-politicas-ia-2026-10.xlsx
+++ b/public/levantamentos/politicas-ia/base-politicas-ia-2026-10.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="1" r:id="R66e10773eb1949a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livro de códigos" sheetId="2" r:id="Rb0051a8e674b4e75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base" sheetId="1" r:id="Rb61b2e9b7c0941aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livro de códigos" sheetId="2" r:id="R19f128aff3444009"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1437,10 +1437,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L22" t="str">
-        <x:v>https://www.sbc.org.br/wp-content/uploads/2024/07/Revis-o-e-atualiza-o-do-C-digo-de-Conduta-para-Autores_Resolucao_2024-001-1.pdf</x:v>
+        <x:v>https://sol.sbc.org.br/index.php/indice/conduta</x:v>
       </x:c>
       <x:c r="M22" t="str">
-        <x:v>Código de Conduta 2024: declarar explicitamente no trabalho.</x:v>
+        <x:v>Código de Conduta para Autores, de 28 de fevereiro de 2024, aplicável aos eventos e publicações realizados ou apoiados pela SBC. Uso de IA para gerar, escrever ou revisar conteúdo deve ser explicitado no trabalho, em Agradecimentos, metodologia ou seção definida pelo template; listar ferramentas e usos, inclusive textos, tabelas e gráficos. IA não é autora e a responsabilidade pelo conteúdo e plágio permanece humana. O código não define regra específica de IA para pareceristas nem regime autônomo de imagens; não inferir permissão para esses papéis e usos.</x:v>
       </x:c>
       <x:c r="N22" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -1652,16 +1652,16 @@
         <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J27" t="str">
-        <x:v>Permitidas c/ declaração</x:v>
+        <x:v>Restritas</x:v>
       </x:c>
       <x:c r="K27" t="str">
         <x:v>P</x:v>
       </x:c>
       <x:c r="L27" t="str">
-        <x:v>https://geoscientist.online/sections/news/ai-in-publishing-geological-society/</x:v>
+        <x:v>https://www.lyellcollection.org/publishing-hub/ai-in-publishing</x:v>
       </x:c>
       <x:c r="M27" t="str">
-        <x:v>Revisores confirmam não envio a LLMs.</x:v>
+        <x:v>Orientação de fevereiro de 2026: edição estilística é dispensada de declaração; geração substantiva de texto é permitida e declarada nos Agradecimentos. Uso na concepção ou pesquisa é descrito em Métodos. A submissão exige informar uso ou não uso. A tabela de integridade classifica como inaceitáveis gerar dados, fabricar resultados, manipular figuras e escrever código para análise nova; não generalizar isso como permissão irrestrita de métodos. Produção de imagens requer declaração conforme o uso, sem fabricar evidência. Revisores não podem enviar manuscritos a LLMs; admitem-se usos auxiliares, como edição gramatical do parecer, com verificação humana. IA não pode ser autora ou revisora nominal.</x:v>
       </x:c>
       <x:c r="N27" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -1684,27 +1684,29 @@
       <x:c r="E28" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F28"/>
+      <x:c r="F28" t="n">
+        <x:v>2024</x:v>
+      </x:c>
       <x:c r="G28" t="str">
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H28" t="str">
-        <x:v>Métodos</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I28" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J28" t="str">
         <x:v>Permitidas c/ declaração</x:v>
       </x:c>
       <x:c r="K28" t="str">
-        <x:v>S</x:v>
+        <x:v>P</x:v>
       </x:c>
       <x:c r="L28" t="str">
-        <x:v>https://policycheck.tools.biorender.com/journal/journal-of-climate</x:v>
+        <x:v>https://www.ametsoc.org/ams/publications/ethical-guidelines-and-ams-policies/author-disclosure-and-obligations/</x:v>
       </x:c>
       <x:c r="M28" t="str">
-        <x:v>Fonte secundária.</x:v>
+        <x:v>American Meteorological Society: cláusula de autores adotada em janeiro de 2024. Uso substantivo de IA na escrita, imagens/gráficos ou coleta/análise de dados deve identificar ferramenta e uso nas seções apropriadas de dados, métodos ou materiais; autores humanos respondem integralmente pelo conteúdo. Revisores não podem avaliar manuscritos ou gerar pareceres com IA nem fazer upload de qualquer parte, mesmo em ferramenta dita segura. A única exceção expressa é editar a linguagem e a clareza do próprio parecer, declarando esse uso no relatório. Não confundir esta AMS com a American Mathematical Society.</x:v>
       </x:c>
       <x:c r="N28" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -1899,9 +1901,7 @@
       <x:c r="E33" t="str">
         <x:v>Internacional</x:v>
       </x:c>
-      <x:c r="F33" t="n">
-        <x:v>2026</x:v>
-      </x:c>
+      <x:c r="F33"/>
       <x:c r="G33" t="str">
         <x:v>Permitida</x:v>
       </x:c>
@@ -1921,7 +1921,7 @@
         <x:v>https://www.elsevier.com/about/policies-and-standards/generative-ai-policies-for-journals</x:v>
       </x:c>
       <x:c r="M33" t="str">
-        <x:v>Política Elsevier; guias com captcha.</x:v>
+        <x:v>RSE, ISPRS Journal e JAG foram conferidos separadamente em seus guias oficiais, que remetem expressamente à política Elsevier. Apoio de IA é permitido com supervisão e contribuição intelectual humana; não admite autoria por IA. Declarar ferramenta e finalidade em seção própria antes das referências, desde a primeira submissão; dispensadas ferramentas básicas de gramática/ortografia/referências e assistência de acessibilidade restrita a esse fim. Editores e pareceristas não podem enviar manuscritos inéditos às ferramentas, mas podem aprimorar a estrutura/linguagem do parecer e pesquisar literatura de contexto. RSE/JAG explicitam ilustrações explicativas e visualizações reprodutíveis derivadas de dados, com declaração na legenda e geral; vedam criar/alterar imagens de dados primários, preservada a pesquisa que usa IA como método. ISPRS remete à política geral e não detalha isoladamente esse regime em sua seção de arte. Não foi identificada data normativa nos guias; 2026 era data de consulta, não de publicação da regra.</x:v>
       </x:c>
       <x:c r="N33" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -2043,7 +2043,7 @@
         <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J36" t="str">
-        <x:v>Restritas</x:v>
+        <x:v>Permitidas c/ declaração</x:v>
       </x:c>
       <x:c r="K36" t="str">
         <x:v>H</x:v>
@@ -2052,7 +2052,7 @@
         <x:v>https://taylorandfrancis.com/our-policies/ai-policy/</x:v>
       </x:c>
       <x:c r="M36" t="str">
-        <x:v>Política T&amp;F; instruções bloqueadas.</x:v>
+        <x:v>IJRS (guia atualizado em 29/09/2025), GIScience &amp; Remote Sensing (12/10/2026) e Remote Sensing Letters (14/09/2026) exigem declaração de uso ou não uso de IA na pesquisa e preparação do manuscrito e remetem às regras T&amp;F. Informar ferramenta, versão, finalidade e modo de uso; os guias não fixam uma seção única. A política geral exige revisão humana rigorosa; veda substituir responsabilidades intelectuais. Admite visualizações e ilustrações conceituais declaradas, não fabricação/manipulação de resultados, amostras ou imagens diagnósticas. Pareceristas só podem melhorar a linguagem do próprio parecer, sem upload de manuscritos, análise/resumo automatizado ou geração de avaliação. Consultados os três guias separadamente; a herança não decorre apenas do vínculo comercial.</x:v>
       </x:c>
       <x:c r="N36" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -2183,7 +2183,7 @@
         <x:v>https://www.scielo.br/journal/bcg/about/?ilang=en</x:v>
       </x:c>
       <x:c r="M39" t="str">
-        <x:v>Ausência confirmada na página integral (versão em inglês), 16/10/2026.</x:v>
+        <x:v>Nas instruções integrais disponíveis no SciELO não foi localizada cláusula específica de IA para escrita, declaração, pareceres ou ilustrações. O periódico remete ao Código de Boas Práticas FAPESP de 2014, que estabelece responsabilidade, autoria, integridade de dados e sigilo, sem regime específico de IA generativa nas seções examinadas. O portal de submissões UFPR estava em manutenção. A ausência codificada limita-se a esse corpus normativo acessível; não certifica inexistência de instruções adicionais nem autoriza uso de IA.</x:v>
       </x:c>
       <x:c r="N39" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -2251,9 +2251,7 @@
       <x:c r="E41" t="str">
         <x:v>Brasil</x:v>
       </x:c>
-      <x:c r="F41" t="n">
-        <x:v>2025</x:v>
-      </x:c>
+      <x:c r="F41"/>
       <x:c r="G41" t="str">
         <x:v>Sem regra</x:v>
       </x:c>
@@ -2270,10 +2268,10 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="L41" t="str">
-        <x:v>https://proceedings.science/sbsr-2025/submission-guidelines?lang=en</x:v>
+        <x:v>https://proceedings.science/cfp/sbsr-2027?lang=pt-br</x:v>
       </x:c>
       <x:c r="M41" t="str">
-        <x:v>Sem regra no XXI SBSR; sem política do INPE localizada.</x:v>
+        <x:v>As normas de artigos do XXII SBSR, edição abril de 2027 já aberta à submissão em 2026, não contêm cláusula específica de IA para redação, declaração, pareceres ou imagens. Exigem originalidade, rigor dos dados, autoria correta e análise por comitê independente. A ausência é delimitada a essas normas PT/EN; não constitui permissão implícita nem política institucional de IA do INPE. As versões divergem no prazo de submissão e a inglesa contém referência residual à edição XXI; a página portuguesa identifica a edição e a prorrogação atuais. Ano da edição não foi tratado como data de publicação da norma.</x:v>
       </x:c>
       <x:c r="N41" t="str">
         <x:v>Ciências Exatas e da Terra</x:v>
@@ -2485,10 +2483,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L46" t="str">
-        <x:v>https://academic.oup.com/PLCELL/pages/General-Instructions</x:v>
+        <x:v>https://academic.oup.com/plcell/pages/author-guidelines</x:v>
       </x:c>
       <x:c r="M46" t="str">
-        <x:v>Carta + Métodos/Agradecimentos; triagem da lista de autores.</x:v>
+        <x:v>Escopo: The Plant Cell, não toda a ASPB. As instruções permitem assistência de IA em conteúdo, imagens, código, dados e tradução sob responsabilidade humana; a IA não pode figurar como autora. Declarar na carta ao editor e em Métodos ou Agradecimentos. Imagens de dados devem representar fielmente os originais, sem inserir, remover ou ocultar características; permissão condicionada de imagens não autoriza fabricar evidência. As seções de revisão e a norma OUP expressamente vinculada exigem sigilo e tratam de conduta, mas não contêm ali uma cláusula específica de IAG para pareceristas; Não trata não significa permissão. Não extrapolar esta página para outros periódicos da sociedade.</x:v>
       </x:c>
       <x:c r="N46" t="str">
         <x:v>Ciências Biológicas</x:v>
@@ -2511,7 +2509,9 @@
       <x:c r="E47" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F47"/>
+      <x:c r="F47" t="n">
+        <x:v>2026</x:v>
+      </x:c>
       <x:c r="G47" t="str">
         <x:v>Restrita</x:v>
       </x:c>
@@ -2519,10 +2519,10 @@
         <x:v>Agradecimentos</x:v>
       </x:c>
       <x:c r="I47" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J47" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Restritas</x:v>
       </x:c>
       <x:c r="K47" t="str">
         <x:v>P</x:v>
@@ -2531,7 +2531,7 @@
         <x:v>https://www.jneurosci.org/content/information-authors</x:v>
       </x:c>
       <x:c r="M47" t="str">
-        <x:v>IA para edição de linguagem.</x:v>
+        <x:v>As instruções de setembro de 2026 permitem IA para edição de linguagem e exigem declarar sua utilização nos Agradecimentos já na submissão. Essa permissão de edição não foi ampliada a geração autônoma do conteúdo científico. As regras SfN, expressamente adotadas pelo periódico, vedam compartilhar manuscritos ou informação confidencial com IA. Condicionado codifica essa vedação de upload: a norma não concede ali autorização expressa para editar pareceres nem enuncia proibição literal de qualquer uso auxiliar. Imagens não podem ter características seletivamente introduzidas, ocultadas, deslocadas ou removidas; ajustes devem ser uniformes e transparentes, com preservação do original. Essas exigências de integridade visual não constituem permissão geral para ilustrações sintéticas.</x:v>
       </x:c>
       <x:c r="N47" t="str">
         <x:v>Ciências Biológicas</x:v>
@@ -2554,14 +2554,12 @@
       <x:c r="E48" t="str">
         <x:v>Internacional</x:v>
       </x:c>
-      <x:c r="F48" t="n">
-        <x:v>2026</x:v>
-      </x:c>
+      <x:c r="F48"/>
       <x:c r="G48" t="str">
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H48" t="str">
-        <x:v>Seção própria</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I48" t="str">
         <x:v>Condicionado</x:v>
@@ -2575,7 +2573,9 @@
       <x:c r="L48" t="str">
         <x:v>https://www.cell.com/cell/information-for-authors/journal-policies</x:v>
       </x:c>
-      <x:c r="M48"/>
+      <x:c r="M48" t="str">
+        <x:v>A Cell admite assistência, agentes e deep research sob controle humano e limites Elsevier. Uso na preparação exige seção própria após a declaração de interesses; ferramentas básicas de gramática, ortografia e referências e ausência de uso dispensam declaração. IA na pesquisa é descrita em Métodos/STAR Methods e na declaração. Ilustrações explicativas são admitidas com legenda e declaração; visualizações devem derivar dos dados e ser reproduzíveis. IA não pode criar ou alterar imagens experimentais/observacionais, nem gerar arte de capa; ferramentas gerais são vedadas para resumos gráficos. Na revisão, adota expressamente as salvaguardas Elsevier: não enviar manuscrito nem delegar avaliação, com assistência auxiliar condicionada. Sem data explícita da norma.</x:v>
+      </x:c>
       <x:c r="N48" t="str">
         <x:v>Ciências Biológicas</x:v>
       </x:c>
@@ -2597,9 +2597,7 @@
       <x:c r="E49" t="str">
         <x:v>Internacional</x:v>
       </x:c>
-      <x:c r="F49" t="n">
-        <x:v>2025</x:v>
-      </x:c>
+      <x:c r="F49"/>
       <x:c r="G49" t="str">
         <x:v>Permitida</x:v>
       </x:c>
@@ -2616,10 +2614,10 @@
         <x:v>H</x:v>
       </x:c>
       <x:c r="L49" t="str">
-        <x:v>https://www.wiley.com/en-us/publishing/article/ai-guidelines</x:v>
+        <x:v>https://onlinelibrary.wiley.com/page/journal/13652486/homepage/forauthors.html</x:v>
       </x:c>
       <x:c r="M49" t="str">
-        <x:v>Política Wiley.</x:v>
+        <x:v>GCB admite desenvolvimento de texto assistido sob responsabilidade humana, sem autoria da IA; pede descrição detalhada em Métodos ou Agradecimentos e dispensa correção ortográfica, gramatical e edição geral. A decisão de adequação é do editor. A instrução do título remete expressamente à confidencialidade Wiley: não enviar manuscritos, figuras ou tabelas a IA; melhoria do parecer exige declaração. A orientação geral Wiley admite ilustração e visualização com salvaguardas de integridade e restrições a fotografias. Regras operacionais de cada imagem devem ser confirmadas com o editor; apoio na escrita não autoriza criar dados. Data da versão normativa não indicada.</x:v>
       </x:c>
       <x:c r="N49" t="str">
         <x:v>Ciências Biológicas</x:v>
@@ -2650,7 +2648,7 @@
         <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I50" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J50" t="str">
         <x:v>Restritas</x:v>
@@ -2659,9 +2657,11 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L50" t="str">
-        <x:v>https://peerj.com/about/policies-and-procedures/</x:v>
-      </x:c>
-      <x:c r="M50"/>
+        <x:v>https://peerj.com/journals/peerj/policies/#generative-ai</x:v>
+      </x:c>
+      <x:c r="M50" t="str">
+        <x:v>Política no portal PeerJ, com remissão expressa à norma de IA Taylor &amp; Francis: IA não é autora; declarar nome, versão, finalidade e uso em Métodos ou Agradecimentos. Revisão linguística e tradução exigem verificação humana, declaração e conservação das versões originais e alteradas. Admite visualizações de dados com registros dos prompts, direitos e declaração na legenda; veda gerar/manipular imagens de resultados científicos ou clínicos. Na norma vinculada, pareceristas não podem enviar manuscritos/informações inéditas, analisar/resumir a submissão ou gerar a avaliação; podem apenas melhorar a linguagem de seu parecer. O sigilo também consta da própria página PeerJ. Não presumir que toda aplicação de IA ou toda imagem seja permitida.</x:v>
+      </x:c>
       <x:c r="N50" t="str">
         <x:v>Ciências Biológicas</x:v>
       </x:c>
@@ -2773,10 +2773,10 @@
       </x:c>
       <x:c r="F53"/>
       <x:c r="G53" t="str">
-        <x:v>Sem regra</x:v>
+        <x:v>Restrita</x:v>
       </x:c>
       <x:c r="H53" t="str">
-        <x:v>—</x:v>
+        <x:v>Não especifica</x:v>
       </x:c>
       <x:c r="I53" t="str">
         <x:v>Não trata</x:v>
@@ -2785,13 +2785,13 @@
         <x:v>Não trata</x:v>
       </x:c>
       <x:c r="K53" t="str">
-        <x:v>A</x:v>
+        <x:v>P</x:v>
       </x:c>
       <x:c r="L53" t="str">
-        <x:v>https://www.scielo.br/journal/abb/about/</x:v>
+        <x:v>https://acta.botanica.org.br/author-guidelines/</x:v>
       </x:c>
       <x:c r="M53" t="str">
-        <x:v>Ausência confirmada nas versões pt e en (página integral, 16/10/2026).</x:v>
+        <x:v>As instruções próprias permitem IA generativa somente para melhorar legibilidade e linguagem, sob revisão e responsabilidade humanas. Vedam gerar ou alterar dados, resultados e conclusões e atribuir autoria à IA. Todo uso deve ser declarado no manuscrito, com ferramenta, modelo/versão e data; não fixam seção única. Não foi encontrada cláusula específica de IA para pareceristas nem um regime próprio de geração de ilustrações nas seções examinadas; a proibição de fabricar dados permanece. A página própria resolve a lacuna da descrição histórica baseada no SciELO. Sem data de edição normativa explícita.</x:v>
       </x:c>
       <x:c r="N53" t="str">
         <x:v>Ciências Biológicas</x:v>
@@ -2945,29 +2945,27 @@
       <x:c r="E57" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F57" t="n">
-        <x:v>2024</x:v>
-      </x:c>
+      <x:c r="F57"/>
       <x:c r="G57" t="str">
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H57" t="str">
-        <x:v>Submissão/carta</x:v>
+        <x:v>Não especifica</x:v>
       </x:c>
       <x:c r="I57" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Vedado</x:v>
       </x:c>
       <x:c r="J57" t="str">
         <x:v>Não trata</x:v>
       </x:c>
       <x:c r="K57" t="str">
-        <x:v>S</x:v>
+        <x:v>P</x:v>
       </x:c>
       <x:c r="L57" t="str">
-        <x:v>https://www.asce.org/publications-and-news/civil-engineering-source/civil-engineering-magazine/issues/magazine-issue/article/2024/03/relying-on-generative-ai-in-scholarly-work-has-its-pitfalls</x:v>
+        <x:v>https://ascelibrary.org/author-center/ai-policy</x:v>
       </x:c>
       <x:c r="M57" t="str">
-        <x:v>Fonte institucional secundária.</x:v>
+        <x:v>A política normativa impede autoria de IA e exige informar se ferramentas de IA foram usadas na criação ou preparação do manuscrito; a ASCE pode exigir detalhes adicionais. A declaração de que não aceita autores não humanos não foi convertida em proibição universal de assistência a autores humanos. A página não fixa seção única para a declaração. Revisores não devem usar LLMs ou IA nem para avaliar manuscritos nem para preparar comentários; as instruções de proceedings repetem essa vedação. Não foi localizada regra específica de IA para imagens nessa política; isso não autoriza fabricar ou manipular dados. Sem data normativa explícita.</x:v>
       </x:c>
       <x:c r="N57" t="str">
         <x:v>Engenharias</x:v>
@@ -3080,7 +3078,9 @@
       <x:c r="E60" t="str">
         <x:v>Brasil</x:v>
       </x:c>
-      <x:c r="F60"/>
+      <x:c r="F60" t="n">
+        <x:v>2025</x:v>
+      </x:c>
       <x:c r="G60" t="str">
         <x:v>Sem regra</x:v>
       </x:c>
@@ -3097,10 +3097,10 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="L60" t="str">
-        <x:v>https://www.scielo.br/journal/esa/about/</x:v>
+        <x:v>https://www.abes-dn.org.br/wp-content/uploads/2025/09/Guidelines-ESA-Journal_Aug_25.pdf</x:v>
       </x:c>
       <x:c r="M60" t="str">
-        <x:v>Ausência confirmada na página integral, 16/10/2026.</x:v>
+        <x:v>O regulamento oficial completo de agosto de 2025, ligado pela ABES, não contém cláusula específica de IA para escrita, declaração, revisão ou imagens. Exige originalidade, métodos reproduzíveis, referências, origem obrigatória das figuras e responsabilidade dos autores; prevê avaliação humana por consultores e editores. A ausência codificada se limita a esse regulamento e às instruções SciELO examinadas, não significa autorização implícita de IA nem comprova inexistência de outras orientações editoriais.</x:v>
       </x:c>
       <x:c r="N60" t="str">
         <x:v>Engenharias</x:v>
@@ -3213,9 +3213,7 @@
       <x:c r="E63" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F63" t="n">
-        <x:v>2026</x:v>
-      </x:c>
+      <x:c r="F63"/>
       <x:c r="G63" t="str">
         <x:v>Permitida</x:v>
       </x:c>
@@ -3235,7 +3233,7 @@
         <x:v>https://www.nejm.org/about-nejm/editorial-policies</x:v>
       </x:c>
       <x:c r="M63" t="str">
-        <x:v>Carta + trabalho; IA generativa vedada em imagens médicas.</x:v>
+        <x:v>O NEJM incorpora expressamente regras ICMJE para a preparação do trabalho: declarar na submissão, tanto na carta quanto no manuscrito, ferramentas e conteúdo produzido; revisar a exatidão, originalidade e referências, sem autoria de IA nem citação de geração sintética como fonte primária. A seção de imagens veda introduzir, mover, remover ou ocultar características e exige declarar ajustes, preservar metadados e não distorcer o original; não equivale a veto genérico de toda ilustração. Na política examinada não foi localizada regra específica de IA para pareceristas, embora sejam descritos avaliação humana e apoio editorial supervisionado. Não há data explícita desta versão normativa.</x:v>
       </x:c>
       <x:c r="N63" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -3353,13 +3351,13 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H66" t="str">
-        <x:v>Submissão/carta</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I66" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Vedado</x:v>
       </x:c>
       <x:c r="J66" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Restritas</x:v>
       </x:c>
       <x:c r="K66" t="str">
         <x:v>P</x:v>
@@ -3368,7 +3366,7 @@
         <x:v>https://www.thelancet.com/editorial-policies</x:v>
       </x:c>
       <x:c r="M66" t="str">
-        <x:v>Restrição por tipo de artigo.</x:v>
+        <x:v>Instruções de agosto/2026: permite apoio à preparação de artigos, com verificação humana e declaração própria ao final do manuscrito (ferramenta, versão, finalidade e supervisão); IA na pesquisa vai em Métodos. Checagens básicas de gramática, ortografia e pontuação são dispensadas na regra geral. Exceções: World Report e Perspectives vedam IA; Comments e Correspondence só admitem gramática/ortografia, com declaração, sem tradução, novos argumentos, resumos ou referências. Figuras geradas diretamente limitam-se a demonstrar a tecnologia em contextos específicos; sugerir conceitos não equivale a fabricar imagem factual. Pareceristas não podem usar IA na avaliação científica nem enviar manuscrito ou comentários, mesmo para melhorar linguagem.</x:v>
       </x:c>
       <x:c r="N66" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -3401,7 +3399,7 @@
         <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I67" t="str">
-        <x:v>Vedado</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J67" t="str">
         <x:v>Restritas</x:v>
@@ -3413,7 +3411,7 @@
         <x:v>https://www.ahajournals.org/ai-guidance</x:v>
       </x:c>
       <x:c r="M67" t="str">
-        <x:v>TRUE-AIM para estudos que treinam IA.</x:v>
+        <x:v>A orientação de junho de 2026 admite escrita assistida sob responsabilidade humana, sem autoria da IA. Uso declarado na submissão e nos Agradecimentos; participação no desenho da pesquisa em Métodos. Correção básica de ortografia, gramática e referências é dispensada. Revisores não podem enviar manuscrito, anexos ou comentários completos a IA; admite-se correção básica integrada ao processador de texto. Não se permite criar, remover, ocultar ou alterar dados em imagens de pesquisa. Infográficos editoriais podem usar IA com declaração, mas exemplos sintéticos de dados científicos ou imagens clínicas são proibidos. Treinamento de IA em pesquisa exige formulário TRUE-AIM na primeira revisão.</x:v>
       </x:c>
       <x:c r="N67" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -3444,19 +3442,19 @@
         <x:v>Métodos</x:v>
       </x:c>
       <x:c r="I68" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Vedado</x:v>
       </x:c>
       <x:c r="J68" t="str">
         <x:v>Não trata</x:v>
       </x:c>
       <x:c r="K68" t="str">
-        <x:v>S</x:v>
+        <x:v>P</x:v>
       </x:c>
       <x:c r="L68" t="str">
-        <x:v>https://manusights.com/blog/journal-of-clinical-oncology-ai-policy</x:v>
+        <x:v>https://ascopubs.org/authors/journal-policies</x:v>
       </x:c>
       <x:c r="M68" t="str">
-        <x:v>LLM vedado em editoriais, revisões, cartas etc.</x:v>
+        <x:v>A ASCO exige declarar em Métodos se IA/LLMs foram usados em Original Reports, Clinical Trial Updates ou na pesquisa, informando ferramenta, versão, data de acesso, fabricante e tarefas. Autores humanos permanecem responsáveis. A preparação por IA é vedada em gêneros centrados em opinião/perspectiva, incluindo Review Articles, editoriais e correspondência; portanto, a permissão não é universal. Revisores não podem usar IA para avaliar trabalhos. A seção de IA não apresenta um regime próprio para imagens; aplicam-se as obrigações gerais de originalidade, consentimento e integridade, sem inferir autorização de imagens sintéticas. Ferramentas editoriais de triagem têm exigência de sigilo. Sem data inequívoca da cláusula.</x:v>
       </x:c>
       <x:c r="N68" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -3484,7 +3482,7 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H69" t="str">
-        <x:v>Não especifica</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I69" t="str">
         <x:v>Condicionado</x:v>
@@ -3493,13 +3491,13 @@
         <x:v>Não trata</x:v>
       </x:c>
       <x:c r="K69" t="str">
-        <x:v>S</x:v>
+        <x:v>P</x:v>
       </x:c>
       <x:c r="L69" t="str">
-        <x:v>https://policycheck.tools.biorender.com/publisher/acp</x:v>
+        <x:v>https://www.acpjournals.org/journal/aim/authors5</x:v>
       </x:c>
       <x:c r="M69" t="str">
-        <x:v>Segue ICMJE.</x:v>
+        <x:v>Escopo ACP/Annals of Internal Medicine, não toda a sociedade. Na submissão, atestar uso ou não de tecnologias assistivas, incluindo LLMs e criadores de imagens; se usadas, descrever na carta e no manuscrito. Autoria e responsabilidade são humanas. Não localizada regra específica por modalidade de imagem nesse corpus; a exigência de declaração não autoriza fabricar evidência. A norma desencoraja IA na revisão e proíbe enviar manuscrito, arquivos, descrição ou comentários do parecer a qualquer ferramenta; editores devem abster-se e comunicar eventual uso por escrito à equipe e autores. Comentários de leitores sobre artigos não podem ser produzidos com IA. Não confundir desencorajamento geral com permissão ampla ou vedação literal de todo uso. Ano normativo não indicado.</x:v>
       </x:c>
       <x:c r="N69" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -3522,15 +3520,17 @@
       <x:c r="E70" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F70"/>
+      <x:c r="F70" t="n">
+        <x:v>2026</x:v>
+      </x:c>
       <x:c r="G70" t="str">
-        <x:v>Restrita</x:v>
+        <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H70" t="str">
-        <x:v>Agradecimentos</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I70" t="str">
-        <x:v>Vedado</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J70" t="str">
         <x:v>Restritas</x:v>
@@ -3542,7 +3542,7 @@
         <x:v>https://aacrjournals.org/pages/editorial-policies</x:v>
       </x:c>
       <x:c r="M70" t="str">
-        <x:v>IA só para revisar ou traduzir texto próprio; gerar texto ou imagens novos é 'inappropriate'; revisores vedados. Estudo próprio: 23% dos resumos com IA em 2024.</x:v>
+        <x:v>Política de março de 2026: revisão ou tradução de texto humano deve ser declarada nos Agradecimentos. Geração de conteúdo novo, inclusive texto ou ilustração, exige descrição na carta e no manuscrito; IA empregada na pesquisa é detalhada em Métodos. Permanecem as exigências de integridade dos dados e autoria humana. Pareceristas não podem delegar análise científica, resumir o estudo ou gerar a crítica por IA. O detalhamento admite apoio à literatura, contexto e apresentação do parecer humano, com declaração; material confidencial só pode ser tratado em ambiente comprovadamente fechado, sem violação de direitos. A política não equivale a proibição absoluta de qualquer uso na revisão.</x:v>
       </x:c>
       <x:c r="N70" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -3701,21 +3701,23 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H74" t="str">
-        <x:v>Métodos</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I74" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J74" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Restritas</x:v>
       </x:c>
       <x:c r="K74" t="str">
-        <x:v>P</x:v>
+        <x:v>H</x:v>
       </x:c>
       <x:c r="L74" t="str">
-        <x:v>https://home.liebertpub.com/publications/ai-in-neuroscience/681/for-authors</x:v>
-      </x:c>
-      <x:c r="M74"/>
+        <x:v>https://journals.sagepub.com/author-instructions/ain?mal-proceed=true</x:v>
+      </x:c>
+      <x:c r="M74" t="str">
+        <x:v>O portfólio Mary Ann Liebert migrou para a plataforma Sage em 2026. A fonte histórica de AI in Neuroscience redireciona para instruções que adotam explicitamente a política Sage: assistência de linguagem, gramática e estrutura é dispensada; geração substantiva e IA em métodos são declaradas na submissão e em Métodos ou Agradecimentos. Admitem-se ilustrações representativas e visualizações declaradas, não imagens fabricadas como evidência original. Revisores podem aprimorar a apresentação do próprio parecer, sem enviar manuscrito a IA ou delegar avaliação. A codificação herdada está comprovada para esse título e a política geral indicada; não certifica exceções de cada periódico do portfólio.</x:v>
+      </x:c>
       <x:c r="N74" t="str">
         <x:v>Ciências da Saúde</x:v>
       </x:c>
@@ -3873,22 +3875,22 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H78" t="str">
-        <x:v>Submissão/carta</x:v>
+        <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I78" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J78" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Restritas</x:v>
       </x:c>
       <x:c r="K78" t="str">
         <x:v>P</x:v>
       </x:c>
       <x:c r="L78" t="str">
-        <x:v>https://www.scielo.br/journal/abc/about/</x:v>
+        <x:v>https://abccardiol.org/politica-sobre-o-uso-de-inteligencia-artificial/</x:v>
       </x:c>
       <x:c r="M78" t="str">
-        <x:v>Declarar IA generativa no formulário de submissão; política própria sobre IA (não lida integralmente).</x:v>
+        <x:v>A política própria admite assistência supervisionada e exige declaração do uso substantivo: escrita, tradução e linguagem nos Agradecimentos ou em declaração específica; uso como método em Métodos, com ferramenta, versão, finalidade e validação. IA não pode ser autora nem fabricar dados, referências ou casos clínicos. Ilustrações e esquemas são admitidos com declaração, precisão e direitos preservados; não podem ser apresentados como dados originais nem alterar evidência. Revisores não podem enviar materiais confidenciais a IA externa ou delegar o parecer; assistência limitada aos próprios comentários exige sigilo e responsabilidade, com uso substantivo comunicado ao editor. Página sem data normativa inequívoca; referências de apoio contêm links inconsistentes e não foram usadas como normas de terceiros.</x:v>
       </x:c>
       <x:c r="N78" t="str">
         <x:v>Ciências da Saúde</x:v>
@@ -4194,10 +4196,10 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="L85" t="str">
-        <x:v>https://www.scielo.br/journal/pab/about/#instructions</x:v>
+        <x:v>https://apct.sede.embrapa.br/pab/en/about/submissions</x:v>
       </x:c>
       <x:c r="M85" t="str">
-        <x:v>Ausência confirmada na página integral, 16/10/2026.</x:v>
+        <x:v>Em 17/10/2026, foram examinadas as instruções integrais de submissão no portal PAB/Embrapa, incluindo autoria, estrutura, Métodos, Agradecimentos, avaliação, figuras e checklist, e a versão SciELO. Nessas páginas não foi localizada uma cláusula específica de IA generativa para redação, declaração, pareceristas ou imagens. Há exigências gerais de originalidade, reprodutibilidade, responsabilidade dos autores e identificação da fonte das figuras. Sem regra significa ausência localizada nesse corpus público, não permissão irrestrita nem prova de inexistência em todo documento interno ou edital. Confirmar com a editoria antes da submissão.</x:v>
       </x:c>
       <x:c r="N85" t="str">
         <x:v>Ciências Agrárias</x:v>
@@ -4240,7 +4242,7 @@
         <x:v>https://www.scielo.br/journal/rbcs/about/#instructions</x:v>
       </x:c>
       <x:c r="M86" t="str">
-        <x:v>Ausência confirmada na página integral, 16/10/2026.</x:v>
+        <x:v>Confronto em 17/10/2026 das políticas editoriais e instruções aos autores publicadas pelo periódico em SciELO, incluindo autoria, declaração, revisão, dados e figuras: não localizada cláusula específica de IA generativa nesses quatro eixos. As exigências gerais de originalidade, responsabilidade, revisão por pares, integridade e apresentação de dados continuam aplicáveis. Sem regra/Não trata descrevem apenas o corpus normativo lido, não autorização irrestrita. O portal próprio rbcsjournal.org não pôde ser lido; a conclusão não cobre normas eventualmente adicionais ali.</x:v>
       </x:c>
       <x:c r="N86" t="str">
         <x:v>Ciências Agrárias</x:v>
@@ -4373,7 +4375,7 @@
         <x:v>https://www.scielo.br/journal/rbeaa/about/#instructions</x:v>
       </x:c>
       <x:c r="M89" t="str">
-        <x:v>Ausência confirmada na página integral, 16/10/2026.</x:v>
+        <x:v>Confronto em 17/10/2026 das políticas editoriais e instruções aos autores publicadas pelo periódico em SciELO, incluindo autoria, declaração, revisão, dados e figuras: não localizada cláusula específica de IA generativa nesses quatro eixos. As exigências gerais de originalidade, responsabilidade, revisão por pares, integridade e apresentação de dados continuam aplicáveis. Sem regra/Não trata descrevem apenas o corpus normativo lido, não autorização irrestrita. O portal agriambi.com.br não pôde ser lido; normas adicionais eventualmente disponíveis ali não foram reconfirmadas.</x:v>
       </x:c>
       <x:c r="N89" t="str">
         <x:v>Ciências Agrárias</x:v>
@@ -4487,10 +4489,10 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H92" t="str">
-        <x:v>Não especifica</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="I92" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J92" t="str">
         <x:v>Não trata</x:v>
@@ -4502,7 +4504,7 @@
         <x:v>https://econometricsociety.org/publications/econometrica/editorial-procedures-and-policies</x:v>
       </x:c>
       <x:c r="M92" t="str">
-        <x:v>Usa IA (Refine) na checagem final.</x:v>
+        <x:v>A política de Econometrica admite IA sob responsabilidade do autor, com verificação de resultados, interpretações, privacidade e propriedade intelectual; veda autoria de software. Não prescreve declaração formal específica de IA nem um regime de imagens na seção examinada. As instruções de pareceristas exigem leitura e avaliação independentes, mas admitem organizar comentários, aprimorar clareza e linguagem; o parecer deve refletir o juízo do revisor. A sociedade usa Refine apenas após aceite condicional para checagens técnicas e expositivas, sem treinamento nos manuscritos e sem julgar contribuição ou publicabilidade. Não se inferiu política de outro periódico ou da Wiley. Sem data explícita da cláusula de IA.</x:v>
       </x:c>
       <x:c r="N92" t="str">
         <x:v>Ciências Sociais Aplicadas</x:v>
@@ -4630,9 +4632,11 @@
         <x:v>NL</x:v>
       </x:c>
       <x:c r="L95" t="str">
-        <x:v>https://www.aals.org/</x:v>
-      </x:c>
-      <x:c r="M95"/>
+        <x:v>https://jle.aals.org/home/submissions.html</x:v>
+      </x:c>
+      <x:c r="M95" t="str">
+        <x:v>Busca dirigida no domínio AALS e leitura integral da página Editorial Policy/Submissions do Journal of Legal Education em 17/10/2026. O texto regula responsabilidade dos autores, checagem editorial, avaliação e imagens, mas não apresenta cláusula específica de IAG para escrita, declaração, pareceristas ou geração de figuras. A entrevista publicada pela AALS sobre a política de sala de aula de Berkeley é opinião/relato de outra instituição, não norma editorial AALS. Mantido NL: não foi localizada uma política institucional geral de publicação com IA no corpus examinado; não se declara inexistência universal nem permissão implícita.</x:v>
+      </x:c>
       <x:c r="N95" t="str">
         <x:v>Ciências Sociais Aplicadas</x:v>
       </x:c>
@@ -4707,7 +4711,7 @@
         <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I97" t="str">
-        <x:v>Vedado</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J97" t="str">
         <x:v>Restritas</x:v>
@@ -4716,10 +4720,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L97" t="str">
-        <x:v>https://www.emeraldgrouppublishing.com/publish-with-us/ethics-integrity/research-publishing-ethics</x:v>
+        <x:v>https://www.emerald.com/publish-with-us/pages/publication-ethics</x:v>
       </x:c>
       <x:c r="M97" t="str">
-        <x:v>Copywriting vedado; copy-editing permitido.</x:v>
+        <x:v>A Emerald veda criar texto novo por IA, inclusive resumo e revisão de literatura, mas permite editar e traduzir trabalho humano existente. Uso generativo é descrito em Métodos e Agradecimentos ou seção apropriada, com ferramenta e versão; a dispensa gramatical refere-se a ferramentas não generativas. Revisores não podem enviar manuscritos à IA, avaliar por ela ou delegar decisões; podem somente melhorar a linguagem de seu próprio parecer, declarando ao editor. Ilustrações conceituais e visualizações de dados humanos são permitidas com identificação, precisão e direitos preservados; imagens factuais sintéticas e arte de capa são vedadas. Datas de consulta não foram tomadas como data da norma.</x:v>
       </x:c>
       <x:c r="N97" t="str">
         <x:v>Ciências Sociais Aplicadas</x:v>
@@ -4978,9 +4982,11 @@
         <x:v>NL</x:v>
       </x:c>
       <x:c r="L103" t="str">
-        <x:v>https://www.aera.net/</x:v>
-      </x:c>
-      <x:c r="M103"/>
+        <x:v>https://www.aera.net/Portals/38/docs/About_AERA/CodeOfEthics(1).pdf</x:v>
+      </x:c>
+      <x:c r="M103" t="str">
+        <x:v>Busca dirigida no domínio AERA e confronto, em 17/10/2026, das normas que sua página de publicações vincula: Code of Ethics (2011), especialmente relato/dados, autoria, publicação e revisores, e Publications Manual (2021). Esses documentos estabelecem responsabilidade, integridade e sigilo, mas não fornecem uma regra específica contemporânea de IAG para os quatro eixos. A notícia AERA de fevereiro de 2026 sobre a visão dos editores de AERA Open descreve ambiguidade sobre uso ético, sem estabelecer uma política geral da associação. Mantido NL: política institucional de IA não localizada nesse corpus, não ausência universal; conferir o periódico. Normas NIH divulgadas pela AERA não são regras editoriais AERA.</x:v>
+      </x:c>
       <x:c r="N103" t="str">
         <x:v>Ciências Humanas</x:v>
       </x:c>
@@ -5047,9 +5053,7 @@
       <x:c r="E105" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F105" t="n">
-        <x:v>2025</x:v>
-      </x:c>
+      <x:c r="F105"/>
       <x:c r="G105" t="str">
         <x:v>Sem regra</x:v>
       </x:c>
@@ -5063,13 +5067,13 @@
         <x:v>Não trata</x:v>
       </x:c>
       <x:c r="K105" t="str">
-        <x:v>A</x:v>
+        <x:v>NL</x:v>
       </x:c>
       <x:c r="L105" t="str">
-        <x:v>https://www.historians.org/resource/guiding-principles-for-artificial-intelligence-in-history-education/</x:v>
+        <x:v>https://www.historians.org/resource/statement-on-standards-of-professional-conduct/</x:v>
       </x:c>
       <x:c r="M105" t="str">
-        <x:v>Só ensino; comitê de pesquisa em curso.</x:v>
+        <x:v>Não foi localizada política institucional específica de IA na publicação após busca dirigida e leitura do Statement on Standards of Professional Conduct, revisto em janeiro de 2023. O documento exige integridade de evidências, atribuição de autoria, reconhecimento de assistência e avaliação responsável, mas não codifica IA nos quatro eixos examinados. A orientação de IA para ensino não prova regra editorial, e a notícia histórica de um comitê não confirma seu estado atual. A conclusão é limitada à documentação oficial consultada: não é ausência universal nem permissão, e não substitui instruções do American Historical Review ou de outro periódico.</x:v>
       </x:c>
       <x:c r="N105" t="str">
         <x:v>Ciências Humanas</x:v>
@@ -5151,12 +5155,14 @@
         <x:v>Não trata</x:v>
       </x:c>
       <x:c r="K107" t="str">
-        <x:v>NL</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="L107" t="str">
-        <x:v>https://www.asanet.org/about/asa-code-of-ethics/</x:v>
-      </x:c>
-      <x:c r="M107"/>
+        <x:v>https://www.asanet.org/about/ethics/</x:v>
+      </x:c>
+      <x:c r="M107" t="str">
+        <x:v>A página Ethics vigente (atualização indicada: 05/10/2025) remete ao Code of Ethics de junho/2018. Examinados pesquisa/dados (12), plágio (13), autoria (14), publicação/edição (15), confidencialidade e revisão (10/16): há responsabilidade humana, proibição de fabricar dados e sigilo, mas não regra específica de IA para escrever, declarar, revisar ou gerar imagens. Ausência verificada nesse código, não em todas as revistas ou atividades da ASA; não atribuir automaticamente a política Sage à sociedade. Data de IA permanece desconhecida.</x:v>
+      </x:c>
       <x:c r="N107" t="str">
         <x:v>Ciências Humanas</x:v>
       </x:c>
@@ -5240,9 +5246,11 @@
         <x:v>NL</x:v>
       </x:c>
       <x:c r="L109" t="str">
-        <x:v>https://www.apaonline.org/</x:v>
-      </x:c>
-      <x:c r="M109"/>
+        <x:v>https://www.apaonline.org/page/journalpractices</x:v>
+      </x:c>
+      <x:c r="M109" t="str">
+        <x:v>Após busca oficial dirigida e leitura da declaração de boas práticas de publicação, aprovada em fevereiro de 2022, não foi localizada regra institucional específica de IA para autores, declaração, pareceristas ou imagens. A declaração exige transparência editorial, avaliação pelo juízo profissional, tratamento de conflitos e respeito às instruções do periódico. Não se transformou esse limite documental em autorização de uso nem ausência universal. A APA filosófica não é a associação psicológica; uma regra de editora ou periódico não foi automaticamente atribuída à sociedade.</x:v>
+      </x:c>
       <x:c r="N109" t="str">
         <x:v>Ciências Humanas</x:v>
       </x:c>
@@ -5264,26 +5272,30 @@
       <x:c r="E110" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F110"/>
+      <x:c r="F110" t="n">
+        <x:v>2026</x:v>
+      </x:c>
       <x:c r="G110" t="str">
-        <x:v>Sem regra</x:v>
+        <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H110" t="str">
-        <x:v>—</x:v>
+        <x:v>Submissão/carta</x:v>
       </x:c>
       <x:c r="I110" t="str">
         <x:v>Não trata</x:v>
       </x:c>
       <x:c r="J110" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Permitidas c/ declaração</x:v>
       </x:c>
       <x:c r="K110" t="str">
-        <x:v>NL</x:v>
+        <x:v>P</x:v>
       </x:c>
       <x:c r="L110" t="str">
-        <x:v>https://papers.aarweb.org/units</x:v>
-      </x:c>
-      <x:c r="M110"/>
+        <x:v>https://papers.aarweb.org/sites/default/files/uploads/PAPERS_Submission_Instructions%202026%20_0.pdf</x:v>
+      </x:c>
+      <x:c r="M110" t="str">
+        <x:v>Registro agregado e heterogêneo. Os códigos positivos referem-se à AAR, reuniões de junho e novembro/2026: declarar na proposta, ao submeter, todo conteúdo gerado por IA (texto, imagens, dados etc.); edição não requer citação. Autores respondem por originalidade, exatidão e atribuição; cada unidade pode rejeitar propostas com IA. Vale também para textos completos e apresentações, não apenas o resumo. O manual não define uso por pareceristas. Para SBL Press foram lidos o guia de propostas, Peer-Review Policy e o guia de figuras: nesse corpus não há cláusula específica de IA; regras gerais de revisão, direitos e figuras não equivalem a permissão implícita. Não há política conjunta demonstrada nem extensão automática aos periódicos da SBL.</x:v>
+      </x:c>
       <x:c r="N110" t="str">
         <x:v>Ciências Humanas</x:v>
       </x:c>
@@ -5305,7 +5317,9 @@
       <x:c r="E111" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F111"/>
+      <x:c r="F111" t="n">
+        <x:v>2026</x:v>
+      </x:c>
       <x:c r="G111" t="str">
         <x:v>Vedada</x:v>
       </x:c>
@@ -5322,10 +5336,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L111" t="str">
-        <x:v>https://www.press.uchicago.edu/resource/ai_guidelines.html</x:v>
+        <x:v>https://press.uchicago.edu/resource/ai_guidelines.html</x:v>
       </x:c>
       <x:c r="M111" t="str">
-        <x:v>Proíbe IA para escrever/reescrever ou gerar argumentos.</x:v>
+        <x:v>Norma de livros atualizada em 22 de junho de 2026; periódicos têm regras próprias. Veda usar IA para escrever/reescrever texto ou gerar argumentos; admite pesquisa auxiliar e correção superficial de gramática. Informar todo uso ao editor na submissão e ao leitor no livro, normalmente em Agradecimentos e/ou notas. Proíbe fabricar/alterar ilustrações, inclusive redesenhar mapas, ampliar arquivos de imagem ou adicionar/remover elementos; permite visualizar dados próprios com declaração. Exige pareceres sem assistência e proíbe enviar manuscrito, proposta ou o próprio parecer a IA, mesmo se a ferramenta prometer não reter dados.</x:v>
       </x:c>
       <x:c r="N111" t="str">
         <x:v>Ciências Humanas</x:v>
@@ -5456,7 +5470,7 @@
         <x:v>https://www.scielo.br/journal/rbedu/about/#instructions</x:v>
       </x:c>
       <x:c r="M114" t="str">
-        <x:v>Ausência confirmada na página integral, 16/10/2026.</x:v>
+        <x:v>Nas versões integrais portuguesa e inglesa das instruções disponibilizadas no SciELO não foi localizada cláusula específica de IA para escrita, declaração, revisão por pares ou imagens. Exigem originalidade, rigor, participação efetiva dos autores, atribuição de fontes e identificação da origem de gráficos e imagens. A codificação Sem regra/Não trata limita-se a essas instruções acessíveis, sem afirmar inexistência de normas adicionais ou autorizar uso de IA. A remissão genérica ao COPE não foi tratada como adoção automática de toda política posterior.</x:v>
       </x:c>
       <x:c r="N114" t="str">
         <x:v>Ciências Humanas</x:v>
@@ -5619,7 +5633,7 @@
         <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H118" t="str">
-        <x:v>Múltiplos</x:v>
+        <x:v>Não especifica</x:v>
       </x:c>
       <x:c r="I118" t="str">
         <x:v>Não trata</x:v>
@@ -5633,7 +5647,9 @@
       <x:c r="L118" t="str">
         <x:v>https://www.mla.org/Publications/MLA-Book-Publications/Resources-for-Contributors/Policy-on-Generative-AI</x:v>
       </x:c>
-      <x:c r="M118"/>
+      <x:c r="M118" t="str">
+        <x:v>Política do programa MLA Book Publications: IA não pode ser autora; todo conteúdo gerado por IA — texto, imagens, dados ou outros — deve ser identificado integralmente no manuscrito no momento da submissão, sem seção fixa indicada. Autores respondem por originalidade, exatidão, atribuição e permissões. Imagens dependem também de seleção e revisão editorial e de direitos adequados. As páginas de IA, submissão e imagens examinadas não estabelecem regra específica de uso por pareceristas; Não trata não equivale a autorização. Esta norma de livros não prova a política operacional da PMLA ou de outras publicações.</x:v>
+      </x:c>
       <x:c r="N118" t="str">
         <x:v>Linguística, Letras e Artes</x:v>
       </x:c>
@@ -5715,9 +5731,11 @@
         <x:v>NL</x:v>
       </x:c>
       <x:c r="L120" t="str">
-        <x:v>https://www.collegeart.org/</x:v>
-      </x:c>
-      <x:c r="M120"/>
+        <x:v>https://www.collegeart.org/publications/preparation</x:v>
+      </x:c>
+      <x:c r="M120" t="str">
+        <x:v>Em 17/10/2026 foram lidas as páginas CAA de submissão de The Art Bulletin e Art Journal, as instruções de preparação aplicáveis também a Art Journal Open e a norma de conflito de interesses/sigilo. Elas regulam originalidade, anonimato, citações, direitos e imagens, mas não explicitam ali um regime próprio de IAG nos quatro eixos. A busca dirigida no domínio CAA não identificou uma política institucional geral aplicável a todas as publicações. Mantido NL: limitação do levantamento, não prova de inexistência ou permissão. A remissão do Art Journal ao portal de submissão T&amp;F não foi tratada como adoção automática de todas as regras da editora.</x:v>
+      </x:c>
       <x:c r="N120" t="str">
         <x:v>Linguística, Letras e Artes</x:v>
       </x:c>
@@ -6357,7 +6375,7 @@
         <x:v>Múltiplos</x:v>
       </x:c>
       <x:c r="I135" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J135" t="str">
         <x:v>Restritas</x:v>
@@ -6368,7 +6386,9 @@
       <x:c r="L135" t="str">
         <x:v>https://f1000research.com/about/policies</x:v>
       </x:c>
-      <x:c r="M135"/>
+      <x:c r="M135" t="str">
+        <x:v>Uso responsável de IA como apoio é admitido com verificação humana, segurança e direitos preservados; não pode substituir responsabilidades centrais do pesquisador. Declarar qualquer uso em Métodos ou Agradecimentos, com nome completo, versão, finalidade e modo de uso. Veda geração/manipulação de imagens, figuras e dados originais; a norma inclui gráficos, tabelas e outras representações. Revisores só podem melhorar a linguagem do próprio parecer e não devem enviar arquivos, imagens ou informações do manuscrito a ferramentas de IA. A avaliação e sua integridade permanecem humanas.</x:v>
+      </x:c>
       <x:c r="N135" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6390,7 +6410,9 @@
       <x:c r="E136" t="str">
         <x:v>EUA</x:v>
       </x:c>
-      <x:c r="F136"/>
+      <x:c r="F136" t="n">
+        <x:v>2026</x:v>
+      </x:c>
       <x:c r="G136" t="str">
         <x:v>Permitida</x:v>
       </x:c>
@@ -6409,7 +6431,9 @@
       <x:c r="L136" t="str">
         <x:v>https://www.science.org/content/page/science-journals-editorial-policies</x:v>
       </x:c>
-      <x:c r="M136"/>
+      <x:c r="M136" t="str">
+        <x:v>A tabela de setembro de 2026 distingue tarefas: escrever ou traduzir conteúdo exige Agradecimentos com modelo e versão; código que altera funcionalidade, geração ou análise de dados são descritos em Métodos. Busca de literatura, edição de linguagem e formatação sem alteração funcional são dispensadas. A política geral pede carta e seção pertinente. Figuras ilustrativas geradas ou alteradas por IA são vedadas sem exceção do editor; editar visualização de resultados exige declaração. Revisores podem refinar sua redação em sistema sem retenção/treinamento e declarar ferramenta e uso, nunca enviar manuscrito. A tabela também veda enviar parecer para gerar resposta e enviar manuscrito à IA na etapa de revisão; refinamento linguístico da resposta tem condições próprias.</x:v>
+      </x:c>
       <x:c r="N136" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
       </x:c>
@@ -6584,7 +6608,7 @@
         <x:v>https://ra.sbpcnet.org.br/78RA/wp-content/uploads/2025/12/2_Normas_de_submissao_de_trabalho_78RA.pdf</x:v>
       </x:c>
       <x:c r="M140" t="str">
-        <x:v>Sem regra nas normas da 78ª RA.</x:v>
+        <x:v>Ausência verificada apenas nas Normas de Submissão de Trabalho da 78ª RA (2026), PDF de dez páginas: não há regra específica de IA para redação, declaração, pareceristas ou imagens. O documento exige responsabilidade do autor, consentimento dos coautores, rigor na revisão e respeito aos direitos sobre figuras; isso não constitui autorização implícita para IA. Não extrapolar para todas as publicações ou futuras reuniões da SBPC. O ano identifica a edição do evento, não uma data de norma de IA.</x:v>
       </x:c>
       <x:c r="N140" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -6662,7 +6686,7 @@
         <x:v>Não especifica</x:v>
       </x:c>
       <x:c r="I142" t="str">
-        <x:v>Vedado</x:v>
+        <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J142" t="str">
         <x:v>Não trata</x:v>
@@ -6671,10 +6695,10 @@
         <x:v>P</x:v>
       </x:c>
       <x:c r="L142" t="str">
-        <x:v>https://www.in.gov.br/web/dou/-/portaria-cnpq-n-2.664-de-6-de-marco-de-2026-691779232</x:v>
+        <x:v>https://www.gov.br/cnpq/pt-br/composicao/comissao-de-integridade/diretrizes</x:v>
       </x:c>
       <x:c r="M142" t="str">
-        <x:v>Declarar em qualquer fase; vedado IA em pareceres.</x:v>
+        <x:v>Diretrizes de integridade da pesquisa apoiada pelo CNPq, atualizadas em 13/03/2026: declarar ferramenta e finalidade de IAG em qualquer fase — concepção, redação, análise ou submissão — nos respectivos textos e exposições eletrônicas. É vedado apresentar conteúdo gerado por IAG como se fosse de autoria humana; os pesquisadores respondem integralmente por plágio, inexatidões e integridade dos dados. Para pareceres, a cláusula I.e veda inserir projetos de terceiros nas ferramentas; não é uma proibição textual de toda assistência, nem autorização para delegar a avaliação. A página dos Comitês, complementar, desaconselha IAG na elaboração de pareceres. Não foi localizada nas diretrizes uma cláusula própria para imagens geradas por IA; aplicam-se os deveres gerais de integridade e transparência. O texto integral do DOU não foi recuperado; a descrição acima é limitada às diretrizes oficiais acessíveis, não a uma transcrição integral da Portaria.</x:v>
       </x:c>
       <x:c r="N142" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -6928,7 +6952,7 @@
         <x:v>2023</x:v>
       </x:c>
       <x:c r="G148" t="str">
-        <x:v>Restrita</x:v>
+        <x:v>Permitida</x:v>
       </x:c>
       <x:c r="H148" t="str">
         <x:v>Múltiplos</x:v>
@@ -6937,16 +6961,16 @@
         <x:v>Condicionado</x:v>
       </x:c>
       <x:c r="J148" t="str">
-        <x:v>Não trata</x:v>
+        <x:v>Restritas</x:v>
       </x:c>
       <x:c r="K148" t="str">
         <x:v>P</x:v>
       </x:c>
       <x:c r="L148" t="str">
-        <x:v>https://www.research.pku.edu.cn/docs/2023-12/20231227162417283170.pdf</x:v>
+        <x:v>https://www.most.gov.cn/kjbgz/202312/W020231221582942330036.pdf</x:v>
       </x:c>
       <x:c r="M148" t="str">
-        <x:v>Guia de conduta responsável (dez/2023): proíbe gerar diretamente materiais de candidatura; rotular conteúdo gerado; declarar em Métodos ou Apêndice; revisores só com consentimento do organizador.</x:v>
+        <x:v>Guia MOST de dezembro de 2023, fonte primária ministerial: admite uso responsável de IAG em pesquisa e no processamento de texto, dados e imagens, sob normas de integridade, sigilo e propriedade intelectual. Não permite gerar diretamente materiais de candidatura a projetos. Conteúdo gerado, sobretudo fatos e argumentos, deve ser identificado e seu processo explicado; referências produzidas por IA não podem ser usadas sem verificação. IA não pode figurar como coautora; declarar usos e detalhes em Métodos, apêndice ou local pertinente, com nome, versão e momento de uso. Avaliadores precisam de consentimento prévio do organizador e devem prevenir vazamento; não é uma autorização geral de parecer automatizado. Imagens não podem ocultar, eliminar ou distorcer dados primários, nem substituir a evidência experimental por imagens externas. O código de redação não elimina a vedação específica para propostas.</x:v>
       </x:c>
       <x:c r="N148" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -7032,9 +7056,11 @@
       <x:c r="K150" t="str">
         <x:v>NL</x:v>
       </x:c>
-      <x:c r="L150"/>
+      <x:c r="L150" t="str">
+        <x:v>https://fapesp.br/boaspraticas/2014/FAPESP-Code_of_Good_Scientific_Practice.pdf</x:v>
+      </x:c>
       <x:c r="M150" t="str">
-        <x:v>Nenhuma norma específica localizada.</x:v>
+        <x:v>Agregado preservado, sem política conjunta demonstrada. FAPESP: código de boas práticas de 2014, seções 3.1–3.5 sobre pesquisa, autoria, dados e pareceres. CAPES: Portaria 24/2025 consolidada (alterada pela 354/2025), especialmente art.8, exige qualidade e sigilo; o texto para discussão sobre IA de 2025 declara não representar necessariamente a CAPES e não é norma. FAPEG: RN1/2008 consolidada sobre comissões (arts.4–10), deveres de publicação na RN1/2024 e alteração 3/2026, com índice atualizado em setembro/2026. Não localizadas cláusulas específicas dos quatro eixos de IA nesses corpora e nas buscas oficiais direcionadas. NL não prova inexistência em editais, orientações internas ou normas posteriores; não significa uso autorizado. Conferir cada agência e edital, sem importar automaticamente a regra do CNPq.</x:v>
       </x:c>
       <x:c r="N150" t="str">
         <x:v>Multidisciplinar / transversal</x:v>
@@ -7139,7 +7165,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="4" t="str">
-        <x:v>Base histórica: 16/10/2026; revisão parcial em 17/10/2026: 105/149 registros reconciliados, 85 corrigidos, 44 pendentes. Data de revisão integral não avançou. Histórico: https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-17.json</x:v>
+        <x:v>Base histórica: 16/10/2026; revisão integral em 17/10/2026: 149/149 registros reconciliados, 129 corrigidos, 0 pendentes. A/NL limitam-se aos corpora descritos, não provam ausência universal. Histórico: https://lapig-ufg.github.io/observatorio-ia/levantamentos/politicas-ia/revisao-2026-10-17.json</x:v>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>